<commit_message>
Docs: ASVS - V6,9 with markdowns and updated on the excel file
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\OneDrive\Documentos\VSRepositories\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6C782E-4B8D-4A5C-BDAE-C490CECFF97B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9621B1E2-DBB4-4712-985F-289134AC4511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" tabRatio="500" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" tabRatio="500" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2123" uniqueCount="957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2136" uniqueCount="970">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2936,6 +2936,45 @@
   </si>
   <si>
     <t>No OIDC back-channel logout is implemented. Not applicable in the current scope.</t>
+  </si>
+  <si>
+    <t>All JWT tokens issued by ArcadeHaven will be validated using their digital signature (HMAC-SHA256 or RS256) before any token content is trusted. Spring Security's JWT filter will reject any token with an invalid or missing signature with a 401 response.</t>
+  </si>
+  <si>
+    <t>An algorithm allowlist will be configured in the JWT validation layer. Only HS256 or RS256 will be permitted. The None algorithm will be explicitly rejected. No mixed symmetric/asymmetric support is planned, avoiding key confusion risks.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven uses a single audience (arcadehaven-api), so audience confusion risk is low.</t>
+  </si>
+  <si>
+    <t>JWT tokens will include an aud (audience) claim set to arcadehaven-api. The validation layer will reject any token whose aud claim does not match the expected value.</t>
+  </si>
+  <si>
+    <t>Key material for JWT validation will be pre-configured server-side via environment variables. JWT headers such as jku, x5u, and jwk will be ignored or validated against a strict allowlist to prevent attackers from supplying untrusted key sources.</t>
+  </si>
+  <si>
+    <t>JWT tokens will include exp (expiration) and nbf (not before) claims. The validation layer will reject tokens outside their validity window. Access tokens will have a maximum lifetime of 15 minutes.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven will issue distinct token types (access token, refresh token)</t>
+  </si>
+  <si>
+    <t>No server-side file decompression is performed on user-uploaded files. Zip slip attacks are not applicable in the current scope.</t>
+  </si>
+  <si>
+    <t>Documentation will define permitted file types per upload feature: game images (JPEG, PNG, WebP — max 5MB), game cover art (JPEG, PNG — max 2MB). System-generated files (PDF invoices, TXT activation keys) have no upload surface. The documentation will also specify behaviour when a malicious file is detected (reject with 400, log the event, notify the admin).</t>
+  </si>
+  <si>
+    <t>Maximum file size limits will be enforced at the Spring Boot level via spring.servlet.multipart.max-file-size and spring.servlet.multipart.max-request-size. Requests exceeding the limit will be rejected with a 413 response before processing begins.</t>
+  </si>
+  <si>
+    <t>All uploaded files will be validated by checking the file extension against an allowlist (JPEG, PNG, WebP) and verifying the magic bytes of the file content. Image files will be re-written server-side (via Java ImageIO) to strip any embedded malicious content and confirm the file is a valid image.</t>
+  </si>
+  <si>
+    <t>No compressed file uploads are accepted. Symlink exploitation via zip files is not applicable in the current scope.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven does not accept compressed archive uploads (zip, gz, etc.).</t>
   </si>
 </sst>
 </file>
@@ -5599,7 +5638,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A3" s="14" t="s">
         <v>490</v>
       </c>
@@ -5616,12 +5655,14 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>957</v>
+      </c>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A4" s="19" t="s">
         <v>490</v>
       </c>
@@ -5638,12 +5679,14 @@
         <v>1</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>958</v>
+      </c>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A5" s="14" t="s">
         <v>490</v>
       </c>
@@ -5660,9 +5703,11 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>961</v>
+      </c>
       <c r="H5" s="16"/>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -5679,7 +5724,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A7" s="14" t="s">
         <v>498</v>
       </c>
@@ -5696,12 +5741,14 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>962</v>
+      </c>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A8" s="19" t="s">
         <v>498</v>
       </c>
@@ -5718,12 +5765,14 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>963</v>
+      </c>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" ht="57" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
         <v>498</v>
       </c>
@@ -5740,12 +5789,14 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>960</v>
+      </c>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A10" s="19" t="s">
         <v>498</v>
       </c>
@@ -5762,9 +5813,11 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G10" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>959</v>
+      </c>
       <c r="H10" s="21"/>
     </row>
   </sheetData>
@@ -12937,7 +12990,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A3" s="14" t="s">
         <v>262</v>
       </c>
@@ -12954,9 +13007,11 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>965</v>
+      </c>
       <c r="H3" s="16"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -12990,12 +13045,14 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>966</v>
+      </c>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" ht="114" x14ac:dyDescent="0.45">
       <c r="A6" s="19" t="s">
         <v>266</v>
       </c>
@@ -13012,12 +13069,14 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>967</v>
+      </c>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A7" s="14" t="s">
         <v>266</v>
       </c>
@@ -13034,9 +13093,11 @@
         <v>2</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="16"/>
+        <v>893</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>969</v>
+      </c>
       <c r="H7" s="16"/>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
@@ -13061,7 +13122,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
         <v>266</v>
       </c>
@@ -13078,9 +13139,11 @@
         <v>3</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="16"/>
+        <v>893</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>968</v>
+      </c>
       <c r="H9" s="16"/>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
@@ -13163,7 +13226,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A14" s="14" t="s">
         <v>280</v>
       </c>
@@ -13180,9 +13243,11 @@
         <v>3</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="16"/>
+        <v>893</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>964</v>
+      </c>
       <c r="H14" s="16"/>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -13284,7 +13349,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Docs: ASVS - V3,4,5 with markdowns and updated on the excel file
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\OneDrive\Documentos\VSRepositories\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9621B1E2-DBB4-4712-985F-289134AC4511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E93E8313-F5F9-4DFA-BB53-2798F364AB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" tabRatio="500" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" tabRatio="500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -2776,9 +2776,6 @@
     <t>REST API with no browser-facing interface. Browser feature detection is not applicable.</t>
   </si>
   <si>
-    <t>REST API. No user-facing redirect notifications are applicable.</t>
-  </si>
-  <si>
     <t>uses no client-side technologies. No plugins, Flash, ActiveX, or applets are used.</t>
   </si>
   <si>
@@ -2962,9 +2959,6 @@
     <t>No server-side file decompression is performed on user-uploaded files. Zip slip attacks are not applicable in the current scope.</t>
   </si>
   <si>
-    <t>Documentation will define permitted file types per upload feature: game images (JPEG, PNG, WebP — max 5MB), game cover art (JPEG, PNG — max 2MB). System-generated files (PDF invoices, TXT activation keys) have no upload surface. The documentation will also specify behaviour when a malicious file is detected (reject with 400, log the event, notify the admin).</t>
-  </si>
-  <si>
     <t>Maximum file size limits will be enforced at the Spring Boot level via spring.servlet.multipart.max-file-size and spring.servlet.multipart.max-request-size. Requests exceeding the limit will be rejected with a 413 response before processing begins.</t>
   </si>
   <si>
@@ -2975,6 +2969,12 @@
   </si>
   <si>
     <t>ArcadeHaven does not accept compressed archive uploads (zip, gz, etc.).</t>
+  </si>
+  <si>
+    <t>Documentation will define permitted file types per upload feature: game images (JPEG, PNG, WebP - max 5MB), game cover art (JPEG, PNG - max 2MB). System-generated files (PDF invoices, TXT activation keys) have no upload surface. The documentation will also specify behaviour when a malicious file is detected (reject with 400, log the event, notify the admin).</t>
+  </si>
+  <si>
+    <t>REST API No user-facing redirect notifications are applicable.</t>
   </si>
 </sst>
 </file>
@@ -5658,7 +5658,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -5682,7 +5682,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -5706,7 +5706,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -5744,7 +5744,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -5768,7 +5768,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="H8" s="21"/>
     </row>
@@ -5792,7 +5792,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -5816,7 +5816,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -5918,7 +5918,7 @@
         <v>893</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -5942,7 +5942,7 @@
         <v>893</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -5980,7 +5980,7 @@
         <v>893</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="H6" s="16"/>
     </row>
@@ -6004,7 +6004,7 @@
         <v>893</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="H7" s="21"/>
     </row>
@@ -6028,7 +6028,7 @@
         <v>893</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="H8" s="16"/>
     </row>
@@ -6066,7 +6066,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -6090,7 +6090,7 @@
         <v>892</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -6114,7 +6114,7 @@
         <v>892</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -6138,7 +6138,7 @@
         <v>893</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="H13" s="21"/>
     </row>
@@ -6162,7 +6162,7 @@
         <v>893</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="H14" s="16"/>
     </row>
@@ -6200,7 +6200,7 @@
         <v>893</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="H16" s="16"/>
     </row>
@@ -6224,7 +6224,7 @@
         <v>893</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="H17" s="21"/>
     </row>
@@ -6248,7 +6248,7 @@
         <v>893</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="H18" s="16"/>
     </row>
@@ -6272,7 +6272,7 @@
         <v>893</v>
       </c>
       <c r="G19" s="21" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="H19" s="21"/>
     </row>
@@ -6296,7 +6296,7 @@
         <v>893</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -6320,7 +6320,7 @@
         <v>893</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -6344,7 +6344,7 @@
         <v>893</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -6368,7 +6368,7 @@
         <v>45</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="H23" s="21"/>
     </row>
@@ -6392,7 +6392,7 @@
         <v>45</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="H24" s="16"/>
     </row>
@@ -6416,7 +6416,7 @@
         <v>893</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H25" s="21"/>
     </row>
@@ -6440,7 +6440,7 @@
         <v>893</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -6464,7 +6464,7 @@
         <v>893</v>
       </c>
       <c r="G27" s="21" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H27" s="21"/>
     </row>
@@ -6488,7 +6488,7 @@
         <v>893</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="H28" s="16"/>
     </row>
@@ -6512,7 +6512,7 @@
         <v>893</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="H29" s="21"/>
     </row>
@@ -6536,7 +6536,7 @@
         <v>893</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H30" s="16"/>
     </row>
@@ -6560,7 +6560,7 @@
         <v>893</v>
       </c>
       <c r="G31" s="21" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H31" s="21"/>
     </row>
@@ -6598,7 +6598,7 @@
         <v>893</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H33" s="16"/>
     </row>
@@ -6622,7 +6622,7 @@
         <v>893</v>
       </c>
       <c r="G34" s="21" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="H34" s="21"/>
     </row>
@@ -6646,7 +6646,7 @@
         <v>893</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="H35" s="16"/>
     </row>
@@ -6670,7 +6670,7 @@
         <v>893</v>
       </c>
       <c r="G36" s="21" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="H36" s="21"/>
     </row>
@@ -6694,7 +6694,7 @@
         <v>893</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="H37" s="16"/>
     </row>
@@ -6732,7 +6732,7 @@
         <v>893</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="H39" s="16"/>
     </row>
@@ -6756,7 +6756,7 @@
         <v>893</v>
       </c>
       <c r="G40" s="21" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="H40" s="21"/>
     </row>
@@ -6794,7 +6794,7 @@
         <v>893</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="H42" s="16"/>
     </row>
@@ -6818,7 +6818,7 @@
         <v>893</v>
       </c>
       <c r="G43" s="21" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H43" s="21"/>
     </row>
@@ -6842,7 +6842,7 @@
         <v>893</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="H44" s="16"/>
     </row>
@@ -7634,7 +7634,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -7680,7 +7680,7 @@
         <v>893</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -8590,7 +8590,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -8650,7 +8650,7 @@
         <v>892</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="H6" s="16"/>
     </row>
@@ -8674,7 +8674,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="H7" s="21"/>
     </row>
@@ -8698,7 +8698,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="H8" s="16"/>
     </row>
@@ -8722,7 +8722,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="H9" s="21"/>
     </row>
@@ -8848,7 +8848,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -8894,7 +8894,7 @@
         <v>893</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -12292,7 +12292,7 @@
         <v>893</v>
       </c>
       <c r="G33" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="H33" s="16"/>
     </row>
@@ -12330,7 +12330,7 @@
         <v>893</v>
       </c>
       <c r="G35" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="H35" s="16"/>
     </row>
@@ -12376,7 +12376,7 @@
         <v>893</v>
       </c>
       <c r="G37" t="s">
-        <v>903</v>
+        <v>969</v>
       </c>
       <c r="H37" s="16"/>
     </row>
@@ -12648,7 +12648,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -12774,7 +12774,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -12798,7 +12798,7 @@
         <v>893</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -12836,7 +12836,7 @@
         <v>893</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="H18" s="16"/>
     </row>
@@ -12860,7 +12860,7 @@
         <v>893</v>
       </c>
       <c r="G19" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="H19" s="21"/>
     </row>
@@ -12884,7 +12884,7 @@
         <v>893</v>
       </c>
       <c r="G20" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -12908,7 +12908,7 @@
         <v>893</v>
       </c>
       <c r="G21" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -12990,7 +12990,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="114" x14ac:dyDescent="0.45">
       <c r="A3" s="14" t="s">
         <v>262</v>
       </c>
@@ -13010,7 +13010,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -13048,7 +13048,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -13072,7 +13072,7 @@
         <v>892</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
       <c r="H6" s="21"/>
     </row>
@@ -13096,7 +13096,7 @@
         <v>893</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -13142,7 +13142,7 @@
         <v>893</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -13246,7 +13246,7 @@
         <v>893</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="H14" s="16"/>
     </row>

</xml_diff>

<commit_message>
Docs: Correction of the ASVS name of V17
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\IdeaProjects\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F548C4-0D86-4752-8B9E-96BC7D565BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0138E65F-4073-4D70-9308-CACADDDEF098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -2983,9 +2983,6 @@
     <t>User-supplied data included in log records is sanitised before writing. IV-001 (whitelist validation) ensures input fields contain only expected characters, and IV-003 (output encoding) applies JSON encoding to any user-controlled value before it is embedded in a structured log entry. CRLF injection — where an attacker submits newline characters in a login username, search query, or game description field to forge or split log entries — is specifically addressed by abuse case AC-21.</t>
   </si>
   <si>
-    <t>ArcadeHaven has no audio or video recording functionality. The only document generation in the platform is PDF invoice creation via the iText library (RF-16, RF-26), which processes structured order data from the database, not media streams. There is no SRTP frame handling, no recording pipeline, and no exposure to malformed media payloads.</t>
-  </si>
-  <si>
     <t>ArcadeHaven's cryptographic keys are documented at the requirements level: the JWT signing secret is managed as an environment variable (RNF-23, SC-001), and the BCrypt cost factor is a configurable application parameter (RNF-01). A formal key management lifecycle document covering key generation, storage, rotation schedule, expiry, and revocation — aligned with NIST SP 800-57 — is being produced. The JWT signing key is the highest-priority asset: its compromise would allow forging authentication tokens for any user role.</t>
   </si>
   <si>
@@ -3133,39 +3130,6 @@
     <t>Although a Level 3 requirement, ArcadeHaven's ER-02 control already defines the global exception handler: a Spring @ControllerAdvice / @ExceptionHandler(Exception.class) that intercepts all unhandled exceptions, logs the full detail (stack trace, correlation ID) internally, and returns a generic client response. This handler functions as a last resort handler by design. A formally verified implementation — confirming that no exception class hierarchy escapes the catch-all handler — is being completed as part of the ER-02 implementation review.</t>
   </si>
   <si>
-    <t>ArcadeHaven has no TURN servers and no peer-to-peer infrastructure. All client-server communication is synchronous REST API over HTTPS. The 30 functional requirements (RF-01 to RF-30) define only game catalog browsing, order management, invoice generation, file upload, and library management — none of which involve NAT traversal or peer-to-peer connectivity.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven has no TURN infrastructure and therefore no TURN allocation mechanism that could be exhausted. Resource exhaustion protection in the platform is applied to REST API endpoints via rate limiting (RNF-09) and temporary account lockout (AC-006). These controls target HTTP request flooding, not TURN allocation abuse.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven does not implement DTLS. The platform uses standard TLS for all HTTPS communication (RNF-05). DTLS is specific to UDP-based media transport and has no role in a synchronous REST API over TCP/TLS. Cipher suite configuration is governed by V12 (Secure Communication), which enforces TLS 1.2 or higher across all API endpoints.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven has no media transcoding pipeline. The platform handles two categories of files: game image uploads from publishers (stored as-is on the server file system) and PDF invoices generated server-side using iText. Neither involves audio or video encoding, transcoding, or streaming. File storage is protected by HTTPS during transit and by access controls during retrieval (FO-003, FO-004).</t>
-  </si>
-  <si>
-    <t>ArcadeHaven transmits no RTP or SRTP streams. All communication between clients and the server is HTTP/REST over TLS (RNF-05). The only "media" distributed by the platform are static files (game images, invoices, activation keys) served as HTTP responses — not real-time audio or video streams.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven processes no real-time media streams and has no stream identifier mechanism. Input validation in the platform applies to JSON request bodies, query parameters, path variables, and uploaded file metadata — not to RTP stream identifiers. Input validation is governed by RNF-06, IV-001 (whitelist validation), and IV-002 (parameterised queries).</t>
-  </si>
-  <si>
-    <t>ArcadeHaven has no media server and receives no SRTP traffic. Flood resilience in the platform is applied at the HTTP API layer via rate limiting (RNF-09) and temporary account lockout (AC-006). These controls protect against HTTP request flooding targeting game catalog, order, and library endpoints — not against SRTP or UDP-based media floods.</t>
-  </si>
-  <si>
-    <t>The ClientHello Race condition is specific to DTLS handshake implementations. ArcadeHaven uses only TLS over TCP for HTTPS communication — there is no DTLS handshake in any part of the application. TLS configuration and cipher suite hardening is addressed in V12 (Secure Communication).</t>
-  </si>
-  <si>
-    <t>ArcadeHaven uses no SDP (Session Description Protocol) and performs no media negotiation. Certificate validation in the platform applies to TLS certificates on HTTPS endpoints and to the outbound HTTPS connection to the RAWG API (RF-12). Media negotiation protocols are entirely outside the platform's architecture.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven has no signaling server and implements no signaling protocol (SIP, XMPP, WebRTC signaling, or custom). All communication is synchronous REST API over HTTPS. Rate limiting is applied to REST API endpoints via RNF-09 and AC-006, covering login, game search, order creation, and other high-volume or security-sensitive operations.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven parses no signaling protocol messages. Malformed request handling in the platform applies to JSON request bodies and multipart form data submitted to REST API endpoints, governed by RNF-06 (input validation), IV-001 (server-side whitelist validation), and IV-003 (output sanitisation). There is no signaling layer where protocol-specific malformed message handling would be required.</t>
-  </si>
-  <si>
     <t>Output is mainly JSON responses and server generated files (PDF invoices, activation keys). When writing files to filesystem, untrusted data will be properly escaped or sanitized</t>
   </si>
   <si>
@@ -3464,6 +3428,42 @@
   </si>
   <si>
     <t>Sensitive responses include Cache-Control: no-store to prevent caching by browsers, proxies, and intermediaries.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven does not implement a TURN server or any NAT traversal mechanism. No real-time peer-to-peer communication is used.</t>
+  </si>
+  <si>
+    <t>No TURN server is used. Resource exhaustion via TURN port allocation is not applicable.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven does not use DTLS or any media server. No cryptographic key management for media transport is required.</t>
+  </si>
+  <si>
+    <t>No media server or DTLS-SRTP is used. Not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>No SRTP or RTP media streams are used. Not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>No media server is implemented. Not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>No media server or SRTP traffic is used. Not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>No DTLS implementation is used. ClientHello race condition is not applicable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	No audio or video recording mechanisms are used. Not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>No DTLS certificates or SDP fingerprint validation is used. Not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven does not implement a signaling server or any WebRTC signaling mechanism. Not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>No signaling server is used. Malformed signaling message handling is not applicable to the current project scope.</t>
   </si>
 </sst>
 </file>
@@ -7492,7 +7492,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -7516,7 +7516,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -7598,7 +7598,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="H8" s="16"/>
     </row>
@@ -7622,7 +7622,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="H9" s="21"/>
     </row>
@@ -7646,7 +7646,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -7670,7 +7670,7 @@
         <v>892</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -7694,7 +7694,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -7732,7 +7732,7 @@
         <v>892</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="H14" s="16"/>
     </row>
@@ -7756,7 +7756,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="H15" s="21"/>
     </row>
@@ -7780,7 +7780,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="H16" s="16"/>
     </row>
@@ -7826,7 +7826,7 @@
         <v>893</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="H18" s="16"/>
     </row>
@@ -7864,7 +7864,7 @@
         <v>892</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -7888,7 +7888,7 @@
         <v>892</v>
       </c>
       <c r="G21" s="27" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -7912,7 +7912,7 @@
         <v>892</v>
       </c>
       <c r="G22" s="27" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -7936,7 +7936,7 @@
         <v>892</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="H23" s="21"/>
     </row>
@@ -7974,7 +7974,7 @@
         <v>892</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="H25" s="16"/>
     </row>
@@ -7998,7 +7998,7 @@
         <v>892</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="H26" s="21"/>
     </row>
@@ -8036,7 +8036,7 @@
         <v>892</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="H28" s="16"/>
     </row>
@@ -8060,7 +8060,7 @@
         <v>893</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="H29" s="21"/>
     </row>
@@ -8098,7 +8098,7 @@
         <v>893</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="H31" s="16"/>
     </row>
@@ -8246,7 +8246,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1119</v>
+        <v>1107</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -8352,7 +8352,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1120</v>
+        <v>1108</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -8376,7 +8376,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>1121</v>
+        <v>1109</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -8414,7 +8414,7 @@
         <v>892</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1123</v>
+        <v>1111</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -8438,7 +8438,7 @@
         <v>892</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>1124</v>
+        <v>1112</v>
       </c>
       <c r="H13" s="21"/>
     </row>
@@ -8462,7 +8462,7 @@
         <v>892</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>1122</v>
+        <v>1110</v>
       </c>
       <c r="H14" s="16"/>
     </row>
@@ -8486,7 +8486,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>1125</v>
+        <v>1113</v>
       </c>
       <c r="H15" s="21"/>
     </row>
@@ -8610,7 +8610,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1126</v>
+        <v>1114</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -8758,7 +8758,7 @@
         <v>893</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1127</v>
+        <v>1115</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -8804,7 +8804,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1128</v>
+        <v>1116</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -9010,7 +9010,7 @@
         <v>893</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>1129</v>
+        <v>1117</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -9100,7 +9100,7 @@
         <v>893</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>1130</v>
+        <v>1118</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -9226,7 +9226,7 @@
         <v>893</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1131</v>
+        <v>1119</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -9486,7 +9486,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1132</v>
+        <v>1120</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -9612,7 +9612,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -9636,7 +9636,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -9660,7 +9660,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -9706,7 +9706,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -9744,7 +9744,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -9768,7 +9768,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -9792,7 +9792,7 @@
         <v>892</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="H11" s="16"/>
     </row>
@@ -9838,7 +9838,7 @@
         <v>892</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="H13" s="16"/>
     </row>
@@ -9876,7 +9876,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -9900,7 +9900,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -9924,7 +9924,7 @@
         <v>892</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -9948,7 +9948,7 @@
         <v>892</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="H18" s="21"/>
     </row>
@@ -9972,7 +9972,7 @@
         <v>892</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="H19" s="16"/>
     </row>
@@ -9996,7 +9996,7 @@
         <v>893</v>
       </c>
       <c r="G20" s="21" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="H20" s="21"/>
     </row>
@@ -10020,7 +10020,7 @@
         <v>892</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -10224,7 +10224,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -10262,7 +10262,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -10286,7 +10286,7 @@
         <v>892</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="H6" s="21"/>
     </row>
@@ -10310,7 +10310,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -10358,7 +10358,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -10420,7 +10420,7 @@
         <v>892</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="H12" s="21"/>
     </row>
@@ -10444,7 +10444,7 @@
         <v>892</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="H13" s="16"/>
     </row>
@@ -10468,7 +10468,7 @@
         <v>893</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="H14" s="21"/>
     </row>
@@ -10530,7 +10530,7 @@
         <v>892</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="H17" s="21"/>
     </row>
@@ -10554,7 +10554,7 @@
         <v>893</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="H18" s="16"/>
     </row>
@@ -10592,7 +10592,7 @@
         <v>892</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -10616,7 +10616,7 @@
         <v>892</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -10640,7 +10640,7 @@
         <v>892</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -10664,7 +10664,7 @@
         <v>892</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="H23" s="21"/>
     </row>
@@ -10746,7 +10746,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="150" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>862</v>
       </c>
@@ -10766,11 +10766,11 @@
         <v>893</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1022</v>
+        <v>1121</v>
       </c>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>862</v>
       </c>
@@ -10790,7 +10790,7 @@
         <v>893</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1023</v>
+        <v>1122</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -10808,7 +10808,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>868</v>
       </c>
@@ -10828,11 +10828,11 @@
         <v>893</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>1024</v>
+        <v>1123</v>
       </c>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="150" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>868</v>
       </c>
@@ -10852,11 +10852,11 @@
         <v>893</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>1025</v>
+        <v>1124</v>
       </c>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>868</v>
       </c>
@@ -10876,11 +10876,11 @@
         <v>893</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>1026</v>
+        <v>1125</v>
       </c>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>868</v>
       </c>
@@ -10900,11 +10900,11 @@
         <v>893</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>1027</v>
+        <v>1126</v>
       </c>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>868</v>
       </c>
@@ -10924,11 +10924,11 @@
         <v>893</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1028</v>
+        <v>1127</v>
       </c>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>868</v>
       </c>
@@ -10948,11 +10948,11 @@
         <v>893</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>1029</v>
+        <v>1128</v>
       </c>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>868</v>
       </c>
@@ -10972,11 +10972,11 @@
         <v>893</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>972</v>
+        <v>1129</v>
       </c>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>868</v>
       </c>
@@ -10996,7 +10996,7 @@
         <v>893</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>1030</v>
+        <v>1130</v>
       </c>
       <c r="H13" s="21"/>
     </row>
@@ -11014,7 +11014,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>886</v>
       </c>
@@ -11034,11 +11034,11 @@
         <v>893</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1031</v>
+        <v>1131</v>
       </c>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="150" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>886</v>
       </c>
@@ -11058,7 +11058,7 @@
         <v>893</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1032</v>
+        <v>1132</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -11160,7 +11160,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="29" t="s">
-        <v>1047</v>
+        <v>1035</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -11184,7 +11184,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="30" t="s">
-        <v>1033</v>
+        <v>1021</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -11222,7 +11222,7 @@
         <v>893</v>
       </c>
       <c r="G6" s="29" t="s">
-        <v>1034</v>
+        <v>1022</v>
       </c>
       <c r="H6" s="16"/>
     </row>
@@ -11312,7 +11312,7 @@
         <v>893</v>
       </c>
       <c r="G10" s="29" t="s">
-        <v>1035</v>
+        <v>1023</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -11336,7 +11336,7 @@
         <v>893</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>1036</v>
+        <v>1024</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -11360,7 +11360,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>1037</v>
+        <v>1025</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -11384,7 +11384,7 @@
         <v>893</v>
       </c>
       <c r="G13" s="30" t="s">
-        <v>1038</v>
+        <v>1026</v>
       </c>
       <c r="H13" s="21"/>
     </row>
@@ -11430,7 +11430,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="30" t="s">
-        <v>1039</v>
+        <v>1027</v>
       </c>
       <c r="H15" s="21"/>
     </row>
@@ -11468,7 +11468,7 @@
         <v>893</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>1040</v>
+        <v>1028</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -11536,7 +11536,7 @@
         <v>893</v>
       </c>
       <c r="G20" s="30" t="s">
-        <v>1041</v>
+        <v>1029</v>
       </c>
       <c r="H20" s="21"/>
     </row>
@@ -11560,7 +11560,7 @@
         <v>893</v>
       </c>
       <c r="G21" s="29" t="s">
-        <v>1042</v>
+        <v>1030</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -11628,7 +11628,7 @@
         <v>893</v>
       </c>
       <c r="G24" s="30" t="s">
-        <v>1043</v>
+        <v>1031</v>
       </c>
       <c r="H24" s="21"/>
     </row>
@@ -11652,7 +11652,7 @@
         <v>893</v>
       </c>
       <c r="G25" s="29" t="s">
-        <v>1044</v>
+        <v>1032</v>
       </c>
       <c r="H25" s="16"/>
     </row>
@@ -11698,7 +11698,7 @@
         <v>893</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>1045</v>
+        <v>1033</v>
       </c>
       <c r="H27" s="16"/>
     </row>
@@ -11758,7 +11758,7 @@
         <v>893</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>1046</v>
+        <v>1034</v>
       </c>
       <c r="H30" s="16"/>
     </row>
@@ -11984,7 +11984,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="29" t="s">
-        <v>1048</v>
+        <v>1036</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -12008,7 +12008,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="30" t="s">
-        <v>1049</v>
+        <v>1037</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -12032,7 +12032,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>1050</v>
+        <v>1038</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -12238,7 +12238,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>1051</v>
+        <v>1039</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -12654,7 +12654,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="25" t="s">
-        <v>1053</v>
+        <v>1041</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -12678,7 +12678,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="26" t="s">
-        <v>1054</v>
+        <v>1042</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -12702,7 +12702,7 @@
         <v>45</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>1055</v>
+        <v>1043</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -12726,7 +12726,7 @@
         <v>892</v>
       </c>
       <c r="G18" s="26" t="s">
-        <v>1056</v>
+        <v>1044</v>
       </c>
       <c r="H18" s="21"/>
     </row>
@@ -12750,7 +12750,7 @@
         <v>893</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>1057</v>
+        <v>1045</v>
       </c>
       <c r="H19" s="16"/>
     </row>
@@ -12774,7 +12774,7 @@
         <v>893</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>1058</v>
+        <v>1046</v>
       </c>
       <c r="H20" s="21"/>
     </row>
@@ -12798,7 +12798,7 @@
         <v>893</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>1059</v>
+        <v>1047</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -12822,7 +12822,7 @@
         <v>893</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>1060</v>
+        <v>1048</v>
       </c>
       <c r="H22" s="21"/>
     </row>
@@ -12860,7 +12860,7 @@
         <v>892</v>
       </c>
       <c r="G24" s="25" t="s">
-        <v>1061</v>
+        <v>1049</v>
       </c>
       <c r="H24" s="16"/>
     </row>
@@ -12884,7 +12884,7 @@
         <v>892</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>1062</v>
+        <v>1050</v>
       </c>
       <c r="H25" s="21"/>
     </row>
@@ -12908,7 +12908,7 @@
         <v>892</v>
       </c>
       <c r="G26" s="25" t="s">
-        <v>1063</v>
+        <v>1051</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -12932,7 +12932,7 @@
         <v>893</v>
       </c>
       <c r="G27" s="26" t="s">
-        <v>1064</v>
+        <v>1052</v>
       </c>
       <c r="H27" s="21"/>
     </row>
@@ -12956,7 +12956,7 @@
         <v>893</v>
       </c>
       <c r="G28" s="25" t="s">
-        <v>1065</v>
+        <v>1053</v>
       </c>
       <c r="H28" s="16"/>
     </row>
@@ -12980,7 +12980,7 @@
         <v>893</v>
       </c>
       <c r="G29" s="26" t="s">
-        <v>1066</v>
+        <v>1054</v>
       </c>
       <c r="H29" s="21"/>
     </row>
@@ -13004,7 +13004,7 @@
         <v>893</v>
       </c>
       <c r="G30" s="25" t="s">
-        <v>1067</v>
+        <v>1055</v>
       </c>
       <c r="H30" s="16"/>
     </row>
@@ -13102,7 +13102,7 @@
         <v>893</v>
       </c>
       <c r="G35" t="s">
-        <v>1052</v>
+        <v>1040</v>
       </c>
       <c r="H35" s="16"/>
     </row>
@@ -13296,7 +13296,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1069</v>
+        <v>1057</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -13320,7 +13320,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1068</v>
+        <v>1056</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -13344,7 +13344,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1070</v>
+        <v>1058</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -14206,7 +14206,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1088</v>
+        <v>1076</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -14230,7 +14230,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1087</v>
+        <v>1075</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -14254,7 +14254,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1084</v>
+        <v>1072</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -14292,7 +14292,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1085</v>
+        <v>1073</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -14316,7 +14316,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>1086</v>
+        <v>1074</v>
       </c>
       <c r="H8" s="21"/>
     </row>
@@ -14340,7 +14340,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1089</v>
+        <v>1077</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -14364,7 +14364,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>1090</v>
+        <v>1078</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -14388,7 +14388,7 @@
         <v>892</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>1091</v>
+        <v>1079</v>
       </c>
       <c r="H11" s="16"/>
     </row>
@@ -14412,7 +14412,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>1092</v>
+        <v>1080</v>
       </c>
       <c r="H12" s="21"/>
     </row>
@@ -14436,7 +14436,7 @@
         <v>893</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1093</v>
+        <v>1081</v>
       </c>
       <c r="H13" s="16"/>
     </row>
@@ -14460,7 +14460,7 @@
         <v>892</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>1094</v>
+        <v>1082</v>
       </c>
       <c r="H14" s="21"/>
     </row>
@@ -14484,7 +14484,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1095</v>
+        <v>1083</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -14508,7 +14508,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1096</v>
+        <v>1084</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -14532,7 +14532,7 @@
         <v>892</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1098</v>
+        <v>1086</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -14556,7 +14556,7 @@
         <v>892</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>1097</v>
+        <v>1085</v>
       </c>
       <c r="H18" s="21"/>
     </row>
@@ -14594,7 +14594,7 @@
         <v>892</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>1099</v>
+        <v>1087</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -14618,7 +14618,7 @@
         <v>892</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>1100</v>
+        <v>1088</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -14642,7 +14642,7 @@
         <v>892</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>1101</v>
+        <v>1089</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -14666,7 +14666,7 @@
         <v>892</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>1102</v>
+        <v>1090</v>
       </c>
       <c r="H23" s="21"/>
     </row>
@@ -14792,7 +14792,7 @@
         <v>892</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>1103</v>
+        <v>1091</v>
       </c>
       <c r="H29" s="16"/>
     </row>
@@ -14816,7 +14816,7 @@
         <v>892</v>
       </c>
       <c r="G30" s="21" t="s">
-        <v>1104</v>
+        <v>1092</v>
       </c>
       <c r="H30" s="21"/>
     </row>
@@ -14840,7 +14840,7 @@
         <v>892</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>1105</v>
+        <v>1093</v>
       </c>
       <c r="H31" s="16"/>
     </row>
@@ -14864,7 +14864,7 @@
         <v>892</v>
       </c>
       <c r="G32" s="21" t="s">
-        <v>1106</v>
+        <v>1094</v>
       </c>
       <c r="H32" s="21"/>
     </row>
@@ -14946,7 +14946,7 @@
         <v>892</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>1110</v>
+        <v>1098</v>
       </c>
       <c r="H36" s="16"/>
     </row>
@@ -14970,7 +14970,7 @@
         <v>892</v>
       </c>
       <c r="G37" s="21" t="s">
-        <v>1107</v>
+        <v>1095</v>
       </c>
       <c r="H37" s="21"/>
     </row>
@@ -14994,7 +14994,7 @@
         <v>892</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>1108</v>
+        <v>1096</v>
       </c>
       <c r="H38" s="16"/>
     </row>
@@ -15018,7 +15018,7 @@
         <v>892</v>
       </c>
       <c r="G39" s="21" t="s">
-        <v>1113</v>
+        <v>1101</v>
       </c>
       <c r="H39" s="21"/>
     </row>
@@ -15042,7 +15042,7 @@
         <v>892</v>
       </c>
       <c r="G40" s="16" t="s">
-        <v>1109</v>
+        <v>1097</v>
       </c>
       <c r="H40" s="16"/>
     </row>
@@ -15146,7 +15146,7 @@
         <v>893</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>1111</v>
+        <v>1099</v>
       </c>
       <c r="H45" s="16"/>
     </row>
@@ -15170,7 +15170,7 @@
         <v>892</v>
       </c>
       <c r="G46" s="21" t="s">
-        <v>1112</v>
+        <v>1100</v>
       </c>
       <c r="H46" s="21"/>
     </row>
@@ -15194,7 +15194,7 @@
         <v>892</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>1114</v>
+        <v>1102</v>
       </c>
       <c r="H47" s="16"/>
     </row>
@@ -15312,7 +15312,7 @@
         <v>893</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>1115</v>
+        <v>1103</v>
       </c>
       <c r="H53" s="16"/>
     </row>
@@ -15336,7 +15336,7 @@
         <v>892</v>
       </c>
       <c r="G54" s="21" t="s">
-        <v>1116</v>
+        <v>1104</v>
       </c>
       <c r="H54" s="21"/>
     </row>
@@ -15360,7 +15360,7 @@
         <v>892</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>1117</v>
+        <v>1105</v>
       </c>
       <c r="H55" s="16"/>
     </row>
@@ -15384,7 +15384,7 @@
         <v>893</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>1118</v>
+        <v>1106</v>
       </c>
       <c r="H56" s="21"/>
     </row>
@@ -15486,7 +15486,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1071</v>
+        <v>1059</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -15510,7 +15510,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1072</v>
+        <v>1060</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -15534,7 +15534,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1073</v>
+        <v>1061</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -16058,7 +16058,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1074</v>
+        <v>1062</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -16082,7 +16082,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1075</v>
+        <v>1063</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -16106,7 +16106,7 @@
         <v>893</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1076</v>
+        <v>1064</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -16130,7 +16130,7 @@
         <v>893</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>1077</v>
+        <v>1065</v>
       </c>
       <c r="H6" s="21"/>
     </row>
@@ -16168,7 +16168,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>1078</v>
+        <v>1066</v>
       </c>
       <c r="H8" s="16"/>
     </row>
@@ -16192,7 +16192,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>1079</v>
+        <v>1067</v>
       </c>
       <c r="H9" s="21"/>
     </row>
@@ -16216,7 +16216,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1080</v>
+        <v>1068</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -16240,7 +16240,7 @@
         <v>893</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>1081</v>
+        <v>1069</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -16322,7 +16322,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1082</v>
+        <v>1070</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -16360,7 +16360,7 @@
         <v>893</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1083</v>
+        <v>1071</v>
       </c>
       <c r="H17" s="16"/>
     </row>

</xml_diff>

<commit_message>
Docs: Modification of the V10 OAuth because of the adaption of Keycloak
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\IdeaProjects\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0138E65F-4073-4D70-9308-CACADDDEF098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867FC1B3-C43B-4388-AAE0-8BA869250391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2299" uniqueCount="1133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2298" uniqueCount="1133">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2827,111 +2827,6 @@
     <t>ArcadeHaven does not implement mutual TLS (mTLS) client certificate authentication in Phase 1. Authentication is handled via JWT Bearer tokens.</t>
   </si>
   <si>
-    <t>ArcadeHaven does not use OAuth2 in Phase 1. Tokens are issued and consumed internally. No backend-for-frontend or token forwarding is used.</t>
-  </si>
-  <si>
-    <t>No external authorization server is used. Token values are generated and validated entirely within the ArcadeHaven backend.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven does not implement an OAuth client or authorization code flow in Phase 1.</t>
-  </si>
-  <si>
-    <t>No multiple authorization server interaction is used. Not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>No OAuth client is implemented. Scope management is handled internally via role-based access control</t>
-  </si>
-  <si>
-    <t>Authorization decisions are based on the role claim in the JWT. Spring Security's method-level security (@PreAuthorize) enforces delegated authorization based on token claims.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven acts as its own resource server. JWT tokens include an aud claim set to arcadehaven-api, validated on every request. Tokens not intended for ArcadeHaven will be rejected.</t>
-  </si>
-  <si>
-    <t>The user's unique identifier is extracted from the JWT for access control decisions. No separate introspection endpoint is used.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven does not require specific authentication strength or recentness for resource access beyond standard JWT validation. Not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>Token theft prevention relies on short expiry (15 minutes) and HTTPS enforcement.</t>
-  </si>
-  <si>
-    <t>Refresh tokens will have an absolute expiration (e.g. 7 days), regardless of usage. Sliding expiration will not be used to prevent indefinite session extension.</t>
-  </si>
-  <si>
-    <t>Users will be able to revoke refresh tokens via the logout endpoint (POST /api/auth/logout). A token denylist will be maintained server-side to immediately invalidate revoked tokens.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven does not implement an OAuth authorization server or redirect URI flows in Phase 1.</t>
-  </si>
-  <si>
-    <t>No authorization code flow is implemented. Not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>No authorization codes are issued. Not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>No OAuth grant types are implemented. Access is controlled via internal JWT issuance only.</t>
-  </si>
-  <si>
-    <t>No refresh token replay mitigation via sender-constrained tokens is needed. Refresh tokens will use rotation each use issues a new token and invalidates the previous one.</t>
-  </si>
-  <si>
-    <t>No authorization code flow or PKCE is implemented</t>
-  </si>
-  <si>
-    <t>No dynamic client registration is supported. ArcadeHaven has no external OAuth clients.</t>
-  </si>
-  <si>
-    <t>No confidential OAuth clients are used. ArcadeHaven issues tokens directly to authenticated users, not to external client applications.</t>
-  </si>
-  <si>
-    <t>No OAuth client scope configuration is applicable. Permissions are managed via user roles defined in the JWT claims.</t>
-  </si>
-  <si>
-    <t>No response_mode configuration is applicable. ArcadeHaven does not implement an OAuth authorization server.</t>
-  </si>
-  <si>
-    <t>No authorization code flow or Pushed Authorization Requests (PAR) are used.</t>
-  </si>
-  <si>
-    <t>No server-side OAuth client is implemented. Not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>No external OAuth client authentication is used. Not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven does not implement an OIDC client or consume ID Tokens from an external provider.</t>
-  </si>
-  <si>
-    <t>Sender-constrained (Proof-of-Possession) tokens are out of scope.</t>
-  </si>
-  <si>
-    <t>User identity is uniquely identified via the sub claim (user UUID) in the internally issued JWT. No external OIDC ID Token is used.</t>
-  </si>
-  <si>
-    <t>ArcadeHaven does not act as an OpenID Provider. Not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>No OAuth consent prompts are displayed. Not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>No OAuth consent grants are managed externally. Users can manage their account and revoke sessions via the ArcadeHaven API directly.</t>
-  </si>
-  <si>
-    <t>No external OAuth authorization flows requiring user consent screens are implemented. ArcadeHaven manages permissions internally via role assignment at registration.</t>
-  </si>
-  <si>
-    <t>No external authorization server is used. Issuer confusion attacks are not applicable in the current scope.</t>
-  </si>
-  <si>
-    <t>No external ID Tokens are consumed. Audience validation is performed on internally issued JWTs</t>
-  </si>
-  <si>
-    <t>No OIDC back-channel logout is implemented. Not applicable in the current scope.</t>
-  </si>
-  <si>
     <t>All JWT tokens issued by ArcadeHaven will be validated using their digital signature (HMAC-SHA256 or RS256) before any token content is trusted. Spring Security's JWT filter will reject any token with an invalid or missing signature with a 401 response.</t>
   </si>
   <si>
@@ -3464,6 +3359,111 @@
   </si>
   <si>
     <t>No signaling server is used. Malformed signaling message handling is not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>The frontend communicates with Keycloak directly. No backend-for-frontend token forwarding is used, the Spring Boot backend only validates tokens, never forwards them to other services.</t>
+  </si>
+  <si>
+    <t>Token values are issued exclusively by Keycloak and validated by the Spring Boot resource server using Keycloak's public keys (via JWKS endpoint). No token mixing between different authorization servers occurs.</t>
+  </si>
+  <si>
+    <t>The frontend uses the Authorization Code flow with PKCE (code_challenge / code_verifier). PKCE inherently protects against CSRF-based token request forgery. Additionally, the state parameter will be generated and validated on every authorization request.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven uses a single Keycloak instance as its only authorization server. Mix-up attacks between multiple authorization servers are not applicable in the current scope.</t>
+  </si>
+  <si>
+    <t>The Spring Boot resource server validates the aud claim in every JWT, ensuring only tokens issued for arcadehaven-api are accepted. Tokens issued for other audiences (e.g. Keycloak admin console) will be rejected.</t>
+  </si>
+  <si>
+    <t>Authorization decisions are enforced by Spring Security using @PreAuthorize annotations. The sub, scope, and role claims from the JWT are all evaluated in access control decisions at the method level</t>
+  </si>
+  <si>
+    <t>Users are uniquely identified by the combination of iss (Keycloak issuer URL) and sub (user UUID) claims. This pair is non-reassignable and used as the canonical user identity across the resource server.</t>
+  </si>
+  <si>
+    <t>Standard JWT validation (expiry, signature, audience) is enforced</t>
+  </si>
+  <si>
+    <t>Token theft mitigation relies on short-lived access tokens (15 minutes) and HTTPS enforcement throughout. This may be revisited in a future phase.</t>
+  </si>
+  <si>
+    <t>Keycloak is configured with an explicit allowlist of valid redirect URIs per client, using exact string matching. Wildcard URIs are not permitted.</t>
+  </si>
+  <si>
+    <t>Keycloak enforces single-use authorization codes natively. If a code is reused, Keycloak rejects the request and revokes any previously issued tokens linked to that code.</t>
+  </si>
+  <si>
+    <t>Authorization codes will be configured with a short lifetime (≤ 1 minute) in Keycloak.</t>
+  </si>
+  <si>
+    <t>Only the Authorization Code grant type is enabled for ArcadeHaven clients in Keycloak. Implicit flow (token) and Resource Owner Password Credentials (password) are explicitly disabled.</t>
+  </si>
+  <si>
+    <t>Keycloak will be configured with refresh token rotation, each use of a refresh token issues a new token and invalidates the previous one. If a revoked refresh token is presented, all tokens for that session are revoked immediately</t>
+  </si>
+  <si>
+    <t>PKCE is enforced for all authorization code requests. Keycloak requires a valid code_challenge using S256 method. The plain method is explicitly disallowed. The code_verifier is validated on every token request.</t>
+  </si>
+  <si>
+    <t>Dynamic client registration is not supported in ArcadeHaven. All clients are pre-registered in Keycloak by administrators. No unauthenticated registration endpoint is exposed.</t>
+  </si>
+  <si>
+    <t>Refresh tokens will have an absolute expiration of 7 days, configured in Keycloak. Sliding expiration is disabled to prevent indefinite session extension.</t>
+  </si>
+  <si>
+    <t>Users can revoke sessions and refresh tokens via the Keycloak account management console and via the ArcadeHaven logout endpoint (POST /api/auth/logout), which calls Keycloak's token revocation endpoint.</t>
+  </si>
+  <si>
+    <t>The Spring Boot backend (acting as a confidential client when needed) authenticates to Keycloak using a client_secret. All backend-to-Keycloak calls (token introspection, revocation) use confidential client credentials.</t>
+  </si>
+  <si>
+    <t>Keycloak client configurations will only include the required scopes (openid, profile, email). No unnecessary scopes are assigned to ArcadeHaven clients.</t>
+  </si>
+  <si>
+    <t>Only response_mode=query (default for code flow) is permitted. No other response modes are configured or accepted for ArcadeHaven clients in Keycloak.</t>
+  </si>
+  <si>
+    <t>Pushed Authorization Requests (PAR) are not implemented</t>
+  </si>
+  <si>
+    <t>Sender-constrained access tokens (mTLS or DPoP) are out of scope for Phase 1. Standard bearer tokens are used, protected by HTTPS and short expiry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	ArcadeHaven does not use authorization_details (Rich Authorization Requests). Not applicable in the current scope.</t>
+  </si>
+  <si>
+    <t>Strong client authentication via mTLS or private_key_jwt is not implemented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Users are uniquely identified by the sub claim in the ID Token, which maps to the Keycloak user UUID. This value is non-reassignable within the Keycloak identity provider.</t>
+  </si>
+  <si>
+    <t>This will generate a nonce value on every authentication request and validate it against the nonce claim in the returned ID Token, protecting against ID Token replay attacks.</t>
+  </si>
+  <si>
+    <t>The Spring Boot backend validate the iss claim against a pre-configured Keycloak issuer URL. Any token with a different issuer is rejected, preventing authorization server impersonation.</t>
+  </si>
+  <si>
+    <t>The aud claim in the ID Token is validated against the registered client_id of the ArcadeHaven frontend client, ensuring tokens issued for other clients are rejected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OIDC back-channel logout is not implemented. Session termination relies on refresh token revocation and short-lived access tokens. </t>
+  </si>
+  <si>
+    <t>Keycloak (acting as the OpenID Provider) is configured to only permit code as the response type for ArcadeHaven clients. Implicit flow (token, id_token token) is explicitly disabled.</t>
+  </si>
+  <si>
+    <t>Keycloak validates the id_token_hint parameter on logout requests and requires explicit user confirmation before terminating sessions. Forced logout DoS is mitigated by Keycloak's built-in logout flow validation.</t>
+  </si>
+  <si>
+    <t>Keycloak is configured to prompt users for consent on every authorization request where the client identity cannot be fully assured. For well-known ArcadeHaven clients, consent may be pre-approved at registration, but this is explicitly configured per client.</t>
+  </si>
+  <si>
+    <t>Keycloak's consent screen presents clear information about the requested scopes, the identity of the authorizing application (ArcadeHaven), and the session lifetime. Users see what they are authorizing before approving.</t>
+  </si>
+  <si>
+    <t>Users can review and revoke active sessions and granted consents via the Keycloak account management console (/realms/arcadehaven/account). The ArcadeHaven logout endpoint also triggers full session revocation via Keycloak.</t>
   </si>
 </sst>
 </file>
@@ -6206,7 +6206,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>955</v>
+        <v>920</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -6230,7 +6230,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>956</v>
+        <v>921</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -6254,7 +6254,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>959</v>
+        <v>924</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -6292,7 +6292,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>960</v>
+        <v>925</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -6316,7 +6316,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>961</v>
+        <v>926</v>
       </c>
       <c r="H8" s="21"/>
     </row>
@@ -6340,7 +6340,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>958</v>
+        <v>923</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -6364,7 +6364,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>957</v>
+        <v>922</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -6446,7 +6446,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>508</v>
       </c>
@@ -6463,10 +6463,10 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>920</v>
+        <v>1098</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -6487,10 +6487,10 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>921</v>
+        <v>1099</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -6508,7 +6508,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>514</v>
       </c>
@@ -6528,7 +6528,7 @@
         <v>893</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>922</v>
+        <v>1100</v>
       </c>
       <c r="H6" s="16"/>
     </row>
@@ -6552,7 +6552,7 @@
         <v>893</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>923</v>
+        <v>1101</v>
       </c>
       <c r="H7" s="21"/>
     </row>
@@ -6575,9 +6575,7 @@
       <c r="F8" s="18" t="s">
         <v>893</v>
       </c>
-      <c r="G8" s="16" t="s">
-        <v>924</v>
-      </c>
+      <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6594,7 +6592,7 @@
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
     </row>
-    <row r="10" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>522</v>
       </c>
@@ -6614,11 +6612,11 @@
         <v>892</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>926</v>
+        <v>1102</v>
       </c>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="106.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>522</v>
       </c>
@@ -6638,11 +6636,11 @@
         <v>892</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>925</v>
+        <v>1103</v>
       </c>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>522</v>
       </c>
@@ -6662,7 +6660,7 @@
         <v>892</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>927</v>
+        <v>1104</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -6686,11 +6684,11 @@
         <v>893</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>928</v>
+        <v>1105</v>
       </c>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>522</v>
       </c>
@@ -6710,7 +6708,7 @@
         <v>893</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>929</v>
+        <v>1106</v>
       </c>
       <c r="H14" s="16"/>
     </row>
@@ -6728,7 +6726,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>534</v>
       </c>
@@ -6745,10 +6743,10 @@
         <v>1</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>932</v>
+        <v>1107</v>
       </c>
       <c r="H16" s="16"/>
     </row>
@@ -6769,10 +6767,10 @@
         <v>1</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>933</v>
+        <v>1108</v>
       </c>
       <c r="H17" s="21"/>
     </row>
@@ -6793,14 +6791,14 @@
         <v>1</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>934</v>
+        <v>1109</v>
       </c>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="105.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>534</v>
       </c>
@@ -6817,10 +6815,10 @@
         <v>1</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G19" s="21" t="s">
-        <v>935</v>
+        <v>1110</v>
       </c>
       <c r="H19" s="21"/>
     </row>
@@ -6841,10 +6839,10 @@
         <v>1</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>936</v>
+        <v>1111</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -6865,10 +6863,10 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>937</v>
+        <v>1112</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -6892,7 +6890,7 @@
         <v>893</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>938</v>
+        <v>1113</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -6913,14 +6911,14 @@
         <v>2</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>45</v>
+        <v>892</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>930</v>
+        <v>1114</v>
       </c>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="107.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>534</v>
       </c>
@@ -6937,14 +6935,14 @@
         <v>2</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>45</v>
+        <v>892</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>931</v>
+        <v>1115</v>
       </c>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="65.650000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>534</v>
       </c>
@@ -6961,14 +6959,14 @@
         <v>2</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>939</v>
+        <v>1116</v>
       </c>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>534</v>
       </c>
@@ -6985,10 +6983,10 @@
         <v>2</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>940</v>
+        <v>1117</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -7012,7 +7010,7 @@
         <v>893</v>
       </c>
       <c r="G27" s="21" t="s">
-        <v>941</v>
+        <v>1118</v>
       </c>
       <c r="H27" s="21"/>
     </row>
@@ -7036,11 +7034,11 @@
         <v>893</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>942</v>
+        <v>1119</v>
       </c>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>534</v>
       </c>
@@ -7060,11 +7058,11 @@
         <v>893</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>946</v>
+        <v>1120</v>
       </c>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>534</v>
       </c>
@@ -7084,11 +7082,11 @@
         <v>893</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>943</v>
+        <v>1121</v>
       </c>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>534</v>
       </c>
@@ -7108,7 +7106,7 @@
         <v>893</v>
       </c>
       <c r="G31" s="21" t="s">
-        <v>944</v>
+        <v>1122</v>
       </c>
       <c r="H31" s="21"/>
     </row>
@@ -7143,14 +7141,14 @@
         <v>2</v>
       </c>
       <c r="F33" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>945</v>
+        <v>1124</v>
       </c>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="86.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>568</v>
       </c>
@@ -7167,14 +7165,14 @@
         <v>2</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G34" s="21" t="s">
-        <v>947</v>
+        <v>1123</v>
       </c>
       <c r="H34" s="21"/>
     </row>
-    <row r="35" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="120" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>568</v>
       </c>
@@ -7191,14 +7189,14 @@
         <v>2</v>
       </c>
       <c r="F35" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>952</v>
+        <v>1125</v>
       </c>
       <c r="H35" s="16"/>
     </row>
-    <row r="36" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
         <v>568</v>
       </c>
@@ -7215,10 +7213,10 @@
         <v>2</v>
       </c>
       <c r="F36" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G36" s="21" t="s">
-        <v>953</v>
+        <v>1126</v>
       </c>
       <c r="H36" s="21"/>
     </row>
@@ -7242,7 +7240,7 @@
         <v>893</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>954</v>
+        <v>1127</v>
       </c>
       <c r="H37" s="16"/>
     </row>
@@ -7260,7 +7258,7 @@
       <c r="G38" s="13"/>
       <c r="H38" s="13"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>580</v>
       </c>
@@ -7277,14 +7275,14 @@
         <v>2</v>
       </c>
       <c r="F39" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>948</v>
+        <v>1128</v>
       </c>
       <c r="H39" s="16"/>
     </row>
-    <row r="40" spans="1:8" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="106.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
         <v>580</v>
       </c>
@@ -7301,10 +7299,10 @@
         <v>2</v>
       </c>
       <c r="F40" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G40" s="21" t="s">
-        <v>948</v>
+        <v>1129</v>
       </c>
       <c r="H40" s="21"/>
     </row>
@@ -7322,7 +7320,7 @@
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
     </row>
-    <row r="42" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="138" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
         <v>586</v>
       </c>
@@ -7339,10 +7337,10 @@
         <v>2</v>
       </c>
       <c r="F42" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>951</v>
+        <v>1130</v>
       </c>
       <c r="H42" s="16"/>
     </row>
@@ -7363,14 +7361,14 @@
         <v>2</v>
       </c>
       <c r="F43" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G43" s="21" t="s">
-        <v>949</v>
+        <v>1131</v>
       </c>
       <c r="H43" s="21"/>
     </row>
-    <row r="44" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="111" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
         <v>586</v>
       </c>
@@ -7387,10 +7385,10 @@
         <v>2</v>
       </c>
       <c r="F44" s="18" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>950</v>
+        <v>1132</v>
       </c>
       <c r="H44" s="16"/>
     </row>
@@ -7406,7 +7404,7 @@
       <formula>"Not Applicable"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="F2:F1044" xr:uid="{00000000-0002-0000-0A00-000000000000}">
       <formula1>"Not Started,In Progress,Compliant,Not Applicable"</formula1>
       <formula2>0</formula2>
@@ -7492,7 +7490,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>972</v>
+        <v>937</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -7516,7 +7514,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>973</v>
+        <v>938</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -7598,7 +7596,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>974</v>
+        <v>939</v>
       </c>
       <c r="H8" s="16"/>
     </row>
@@ -7622,7 +7620,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>975</v>
+        <v>940</v>
       </c>
       <c r="H9" s="21"/>
     </row>
@@ -7646,7 +7644,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>976</v>
+        <v>941</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -7670,7 +7668,7 @@
         <v>892</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>977</v>
+        <v>942</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -7694,7 +7692,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>978</v>
+        <v>943</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -7732,7 +7730,7 @@
         <v>892</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>979</v>
+        <v>944</v>
       </c>
       <c r="H14" s="16"/>
     </row>
@@ -7756,7 +7754,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>980</v>
+        <v>945</v>
       </c>
       <c r="H15" s="21"/>
     </row>
@@ -7780,7 +7778,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>981</v>
+        <v>946</v>
       </c>
       <c r="H16" s="16"/>
     </row>
@@ -7826,7 +7824,7 @@
         <v>893</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>982</v>
+        <v>947</v>
       </c>
       <c r="H18" s="16"/>
     </row>
@@ -7864,7 +7862,7 @@
         <v>892</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>983</v>
+        <v>948</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -7888,7 +7886,7 @@
         <v>892</v>
       </c>
       <c r="G21" s="27" t="s">
-        <v>984</v>
+        <v>949</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -7912,7 +7910,7 @@
         <v>892</v>
       </c>
       <c r="G22" s="27" t="s">
-        <v>985</v>
+        <v>950</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -7936,7 +7934,7 @@
         <v>892</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>986</v>
+        <v>951</v>
       </c>
       <c r="H23" s="21"/>
     </row>
@@ -7974,7 +7972,7 @@
         <v>892</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>987</v>
+        <v>952</v>
       </c>
       <c r="H25" s="16"/>
     </row>
@@ -7998,7 +7996,7 @@
         <v>892</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>988</v>
+        <v>953</v>
       </c>
       <c r="H26" s="21"/>
     </row>
@@ -8036,7 +8034,7 @@
         <v>892</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>989</v>
+        <v>954</v>
       </c>
       <c r="H28" s="16"/>
     </row>
@@ -8060,7 +8058,7 @@
         <v>893</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>990</v>
+        <v>955</v>
       </c>
       <c r="H29" s="21"/>
     </row>
@@ -8098,7 +8096,7 @@
         <v>893</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>991</v>
+        <v>956</v>
       </c>
       <c r="H31" s="16"/>
     </row>
@@ -8246,7 +8244,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1107</v>
+        <v>1072</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -8352,7 +8350,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1108</v>
+        <v>1073</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -8376,7 +8374,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>1109</v>
+        <v>1074</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -8414,7 +8412,7 @@
         <v>892</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1111</v>
+        <v>1076</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -8438,7 +8436,7 @@
         <v>892</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>1112</v>
+        <v>1077</v>
       </c>
       <c r="H13" s="21"/>
     </row>
@@ -8462,7 +8460,7 @@
         <v>892</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>1110</v>
+        <v>1075</v>
       </c>
       <c r="H14" s="16"/>
     </row>
@@ -8486,7 +8484,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>1113</v>
+        <v>1078</v>
       </c>
       <c r="H15" s="21"/>
     </row>
@@ -8610,7 +8608,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1114</v>
+        <v>1079</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -8758,7 +8756,7 @@
         <v>893</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1115</v>
+        <v>1080</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -8804,7 +8802,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1116</v>
+        <v>1081</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -9010,7 +9008,7 @@
         <v>893</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>1117</v>
+        <v>1082</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -9100,7 +9098,7 @@
         <v>893</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>1118</v>
+        <v>1083</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -9226,7 +9224,7 @@
         <v>893</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1119</v>
+        <v>1084</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -9486,7 +9484,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1120</v>
+        <v>1085</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -9612,7 +9610,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>992</v>
+        <v>957</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -9636,7 +9634,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>993</v>
+        <v>958</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -9660,7 +9658,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>994</v>
+        <v>959</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -9706,7 +9704,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>995</v>
+        <v>960</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -9744,7 +9742,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>996</v>
+        <v>961</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -9768,7 +9766,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>997</v>
+        <v>962</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -9792,7 +9790,7 @@
         <v>892</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>998</v>
+        <v>963</v>
       </c>
       <c r="H11" s="16"/>
     </row>
@@ -9838,7 +9836,7 @@
         <v>892</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>999</v>
+        <v>964</v>
       </c>
       <c r="H13" s="16"/>
     </row>
@@ -9876,7 +9874,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1000</v>
+        <v>965</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -9900,7 +9898,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1001</v>
+        <v>966</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -9924,7 +9922,7 @@
         <v>892</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1002</v>
+        <v>967</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -9948,7 +9946,7 @@
         <v>892</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>1003</v>
+        <v>968</v>
       </c>
       <c r="H18" s="21"/>
     </row>
@@ -9972,7 +9970,7 @@
         <v>892</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>1004</v>
+        <v>969</v>
       </c>
       <c r="H19" s="16"/>
     </row>
@@ -9996,7 +9994,7 @@
         <v>893</v>
       </c>
       <c r="G20" s="21" t="s">
-        <v>1005</v>
+        <v>970</v>
       </c>
       <c r="H20" s="21"/>
     </row>
@@ -10020,7 +10018,7 @@
         <v>892</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>1006</v>
+        <v>971</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -10224,7 +10222,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1008</v>
+        <v>973</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -10262,7 +10260,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1012</v>
+        <v>977</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -10286,7 +10284,7 @@
         <v>892</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>1011</v>
+        <v>976</v>
       </c>
       <c r="H6" s="21"/>
     </row>
@@ -10310,7 +10308,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1010</v>
+        <v>975</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -10334,7 +10332,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>969</v>
+        <v>934</v>
       </c>
       <c r="H8" s="21"/>
     </row>
@@ -10358,7 +10356,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1009</v>
+        <v>974</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -10396,7 +10394,7 @@
         <v>892</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>970</v>
+        <v>935</v>
       </c>
       <c r="H11" s="16"/>
     </row>
@@ -10420,7 +10418,7 @@
         <v>892</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>1007</v>
+        <v>972</v>
       </c>
       <c r="H12" s="21"/>
     </row>
@@ -10444,7 +10442,7 @@
         <v>892</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1013</v>
+        <v>978</v>
       </c>
       <c r="H13" s="16"/>
     </row>
@@ -10468,7 +10466,7 @@
         <v>893</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>1014</v>
+        <v>979</v>
       </c>
       <c r="H14" s="21"/>
     </row>
@@ -10506,7 +10504,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>971</v>
+        <v>936</v>
       </c>
       <c r="H16" s="16"/>
     </row>
@@ -10530,7 +10528,7 @@
         <v>892</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>1015</v>
+        <v>980</v>
       </c>
       <c r="H17" s="21"/>
     </row>
@@ -10554,7 +10552,7 @@
         <v>893</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>1016</v>
+        <v>981</v>
       </c>
       <c r="H18" s="16"/>
     </row>
@@ -10592,7 +10590,7 @@
         <v>892</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>1017</v>
+        <v>982</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -10616,7 +10614,7 @@
         <v>892</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>1018</v>
+        <v>983</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -10640,7 +10638,7 @@
         <v>892</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>1019</v>
+        <v>984</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -10664,7 +10662,7 @@
         <v>892</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>1020</v>
+        <v>985</v>
       </c>
       <c r="H23" s="21"/>
     </row>
@@ -10766,7 +10764,7 @@
         <v>893</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1121</v>
+        <v>1086</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -10790,7 +10788,7 @@
         <v>893</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1122</v>
+        <v>1087</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -10828,7 +10826,7 @@
         <v>893</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>1123</v>
+        <v>1088</v>
       </c>
       <c r="H6" s="16"/>
     </row>
@@ -10852,7 +10850,7 @@
         <v>893</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>1124</v>
+        <v>1089</v>
       </c>
       <c r="H7" s="21"/>
     </row>
@@ -10876,7 +10874,7 @@
         <v>893</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>1125</v>
+        <v>1090</v>
       </c>
       <c r="H8" s="16"/>
     </row>
@@ -10900,7 +10898,7 @@
         <v>893</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>1126</v>
+        <v>1091</v>
       </c>
       <c r="H9" s="21"/>
     </row>
@@ -10924,7 +10922,7 @@
         <v>893</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1127</v>
+        <v>1092</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -10948,7 +10946,7 @@
         <v>893</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>1128</v>
+        <v>1093</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -10972,7 +10970,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1129</v>
+        <v>1094</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -10996,7 +10994,7 @@
         <v>893</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>1130</v>
+        <v>1095</v>
       </c>
       <c r="H13" s="21"/>
     </row>
@@ -11034,7 +11032,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1131</v>
+        <v>1096</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -11058,7 +11056,7 @@
         <v>893</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1132</v>
+        <v>1097</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -11160,7 +11158,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="29" t="s">
-        <v>1035</v>
+        <v>1000</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -11184,7 +11182,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="30" t="s">
-        <v>1021</v>
+        <v>986</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -11222,7 +11220,7 @@
         <v>893</v>
       </c>
       <c r="G6" s="29" t="s">
-        <v>1022</v>
+        <v>987</v>
       </c>
       <c r="H6" s="16"/>
     </row>
@@ -11312,7 +11310,7 @@
         <v>893</v>
       </c>
       <c r="G10" s="29" t="s">
-        <v>1023</v>
+        <v>988</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -11336,7 +11334,7 @@
         <v>893</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>1024</v>
+        <v>989</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -11360,7 +11358,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>1025</v>
+        <v>990</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -11384,7 +11382,7 @@
         <v>893</v>
       </c>
       <c r="G13" s="30" t="s">
-        <v>1026</v>
+        <v>991</v>
       </c>
       <c r="H13" s="21"/>
     </row>
@@ -11430,7 +11428,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="30" t="s">
-        <v>1027</v>
+        <v>992</v>
       </c>
       <c r="H15" s="21"/>
     </row>
@@ -11468,7 +11466,7 @@
         <v>893</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>1028</v>
+        <v>993</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -11536,7 +11534,7 @@
         <v>893</v>
       </c>
       <c r="G20" s="30" t="s">
-        <v>1029</v>
+        <v>994</v>
       </c>
       <c r="H20" s="21"/>
     </row>
@@ -11560,7 +11558,7 @@
         <v>893</v>
       </c>
       <c r="G21" s="29" t="s">
-        <v>1030</v>
+        <v>995</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -11628,7 +11626,7 @@
         <v>893</v>
       </c>
       <c r="G24" s="30" t="s">
-        <v>1031</v>
+        <v>996</v>
       </c>
       <c r="H24" s="21"/>
     </row>
@@ -11652,7 +11650,7 @@
         <v>893</v>
       </c>
       <c r="G25" s="29" t="s">
-        <v>1032</v>
+        <v>997</v>
       </c>
       <c r="H25" s="16"/>
     </row>
@@ -11698,7 +11696,7 @@
         <v>893</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>1033</v>
+        <v>998</v>
       </c>
       <c r="H27" s="16"/>
     </row>
@@ -11758,7 +11756,7 @@
         <v>893</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>1034</v>
+        <v>999</v>
       </c>
       <c r="H30" s="16"/>
     </row>
@@ -11984,7 +11982,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="29" t="s">
-        <v>1036</v>
+        <v>1001</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -12008,7 +12006,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="30" t="s">
-        <v>1037</v>
+        <v>1002</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -12032,7 +12030,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>1038</v>
+        <v>1003</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -12238,7 +12236,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>1039</v>
+        <v>1004</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -12654,7 +12652,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="25" t="s">
-        <v>1041</v>
+        <v>1006</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -12678,7 +12676,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="26" t="s">
-        <v>1042</v>
+        <v>1007</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -12702,7 +12700,7 @@
         <v>45</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>1043</v>
+        <v>1008</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -12726,7 +12724,7 @@
         <v>892</v>
       </c>
       <c r="G18" s="26" t="s">
-        <v>1044</v>
+        <v>1009</v>
       </c>
       <c r="H18" s="21"/>
     </row>
@@ -12750,7 +12748,7 @@
         <v>893</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>1045</v>
+        <v>1010</v>
       </c>
       <c r="H19" s="16"/>
     </row>
@@ -12774,7 +12772,7 @@
         <v>893</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>1046</v>
+        <v>1011</v>
       </c>
       <c r="H20" s="21"/>
     </row>
@@ -12798,7 +12796,7 @@
         <v>893</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>1047</v>
+        <v>1012</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -12822,7 +12820,7 @@
         <v>893</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>1048</v>
+        <v>1013</v>
       </c>
       <c r="H22" s="21"/>
     </row>
@@ -12860,7 +12858,7 @@
         <v>892</v>
       </c>
       <c r="G24" s="25" t="s">
-        <v>1049</v>
+        <v>1014</v>
       </c>
       <c r="H24" s="16"/>
     </row>
@@ -12884,7 +12882,7 @@
         <v>892</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>1050</v>
+        <v>1015</v>
       </c>
       <c r="H25" s="21"/>
     </row>
@@ -12908,7 +12906,7 @@
         <v>892</v>
       </c>
       <c r="G26" s="25" t="s">
-        <v>1051</v>
+        <v>1016</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -12932,7 +12930,7 @@
         <v>893</v>
       </c>
       <c r="G27" s="26" t="s">
-        <v>1052</v>
+        <v>1017</v>
       </c>
       <c r="H27" s="21"/>
     </row>
@@ -12956,7 +12954,7 @@
         <v>893</v>
       </c>
       <c r="G28" s="25" t="s">
-        <v>1053</v>
+        <v>1018</v>
       </c>
       <c r="H28" s="16"/>
     </row>
@@ -12980,7 +12978,7 @@
         <v>893</v>
       </c>
       <c r="G29" s="26" t="s">
-        <v>1054</v>
+        <v>1019</v>
       </c>
       <c r="H29" s="21"/>
     </row>
@@ -13004,7 +13002,7 @@
         <v>893</v>
       </c>
       <c r="G30" s="25" t="s">
-        <v>1055</v>
+        <v>1020</v>
       </c>
       <c r="H30" s="16"/>
     </row>
@@ -13102,7 +13100,7 @@
         <v>893</v>
       </c>
       <c r="G35" t="s">
-        <v>1040</v>
+        <v>1005</v>
       </c>
       <c r="H35" s="16"/>
     </row>
@@ -13148,7 +13146,7 @@
         <v>893</v>
       </c>
       <c r="G37" t="s">
-        <v>968</v>
+        <v>933</v>
       </c>
       <c r="H37" s="16"/>
     </row>
@@ -13296,7 +13294,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1057</v>
+        <v>1022</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -13320,7 +13318,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1056</v>
+        <v>1021</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -13344,7 +13342,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1058</v>
+        <v>1023</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -13788,7 +13786,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>967</v>
+        <v>932</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -13826,7 +13824,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>963</v>
+        <v>928</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -13850,7 +13848,7 @@
         <v>892</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>964</v>
+        <v>929</v>
       </c>
       <c r="H6" s="21"/>
     </row>
@@ -13874,7 +13872,7 @@
         <v>893</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>966</v>
+        <v>931</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -13920,7 +13918,7 @@
         <v>893</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>965</v>
+        <v>930</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -14024,7 +14022,7 @@
         <v>893</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>962</v>
+        <v>927</v>
       </c>
       <c r="H14" s="16"/>
     </row>
@@ -14206,7 +14204,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1076</v>
+        <v>1041</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -14230,7 +14228,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1075</v>
+        <v>1040</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -14254,7 +14252,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1072</v>
+        <v>1037</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -14292,7 +14290,7 @@
         <v>892</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1073</v>
+        <v>1038</v>
       </c>
       <c r="H7" s="16"/>
     </row>
@@ -14316,7 +14314,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>1074</v>
+        <v>1039</v>
       </c>
       <c r="H8" s="21"/>
     </row>
@@ -14340,7 +14338,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1077</v>
+        <v>1042</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -14364,7 +14362,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>1078</v>
+        <v>1043</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -14388,7 +14386,7 @@
         <v>892</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>1079</v>
+        <v>1044</v>
       </c>
       <c r="H11" s="16"/>
     </row>
@@ -14412,7 +14410,7 @@
         <v>893</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>1080</v>
+        <v>1045</v>
       </c>
       <c r="H12" s="21"/>
     </row>
@@ -14436,7 +14434,7 @@
         <v>893</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1081</v>
+        <v>1046</v>
       </c>
       <c r="H13" s="16"/>
     </row>
@@ -14460,7 +14458,7 @@
         <v>892</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>1082</v>
+        <v>1047</v>
       </c>
       <c r="H14" s="21"/>
     </row>
@@ -14484,7 +14482,7 @@
         <v>892</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1083</v>
+        <v>1048</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -14508,7 +14506,7 @@
         <v>892</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1084</v>
+        <v>1049</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -14532,7 +14530,7 @@
         <v>892</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1086</v>
+        <v>1051</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -14556,7 +14554,7 @@
         <v>892</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>1085</v>
+        <v>1050</v>
       </c>
       <c r="H18" s="21"/>
     </row>
@@ -14594,7 +14592,7 @@
         <v>892</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>1087</v>
+        <v>1052</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -14618,7 +14616,7 @@
         <v>892</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>1088</v>
+        <v>1053</v>
       </c>
       <c r="H21" s="21"/>
     </row>
@@ -14642,7 +14640,7 @@
         <v>892</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>1089</v>
+        <v>1054</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -14666,7 +14664,7 @@
         <v>892</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>1090</v>
+        <v>1055</v>
       </c>
       <c r="H23" s="21"/>
     </row>
@@ -14792,7 +14790,7 @@
         <v>892</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>1091</v>
+        <v>1056</v>
       </c>
       <c r="H29" s="16"/>
     </row>
@@ -14816,7 +14814,7 @@
         <v>892</v>
       </c>
       <c r="G30" s="21" t="s">
-        <v>1092</v>
+        <v>1057</v>
       </c>
       <c r="H30" s="21"/>
     </row>
@@ -14840,7 +14838,7 @@
         <v>892</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>1093</v>
+        <v>1058</v>
       </c>
       <c r="H31" s="16"/>
     </row>
@@ -14864,7 +14862,7 @@
         <v>892</v>
       </c>
       <c r="G32" s="21" t="s">
-        <v>1094</v>
+        <v>1059</v>
       </c>
       <c r="H32" s="21"/>
     </row>
@@ -14946,7 +14944,7 @@
         <v>892</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>1098</v>
+        <v>1063</v>
       </c>
       <c r="H36" s="16"/>
     </row>
@@ -14970,7 +14968,7 @@
         <v>892</v>
       </c>
       <c r="G37" s="21" t="s">
-        <v>1095</v>
+        <v>1060</v>
       </c>
       <c r="H37" s="21"/>
     </row>
@@ -14994,7 +14992,7 @@
         <v>892</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>1096</v>
+        <v>1061</v>
       </c>
       <c r="H38" s="16"/>
     </row>
@@ -15018,7 +15016,7 @@
         <v>892</v>
       </c>
       <c r="G39" s="21" t="s">
-        <v>1101</v>
+        <v>1066</v>
       </c>
       <c r="H39" s="21"/>
     </row>
@@ -15042,7 +15040,7 @@
         <v>892</v>
       </c>
       <c r="G40" s="16" t="s">
-        <v>1097</v>
+        <v>1062</v>
       </c>
       <c r="H40" s="16"/>
     </row>
@@ -15146,7 +15144,7 @@
         <v>893</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>1099</v>
+        <v>1064</v>
       </c>
       <c r="H45" s="16"/>
     </row>
@@ -15170,7 +15168,7 @@
         <v>892</v>
       </c>
       <c r="G46" s="21" t="s">
-        <v>1100</v>
+        <v>1065</v>
       </c>
       <c r="H46" s="21"/>
     </row>
@@ -15194,7 +15192,7 @@
         <v>892</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>1102</v>
+        <v>1067</v>
       </c>
       <c r="H47" s="16"/>
     </row>
@@ -15312,7 +15310,7 @@
         <v>893</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>1103</v>
+        <v>1068</v>
       </c>
       <c r="H53" s="16"/>
     </row>
@@ -15336,7 +15334,7 @@
         <v>892</v>
       </c>
       <c r="G54" s="21" t="s">
-        <v>1104</v>
+        <v>1069</v>
       </c>
       <c r="H54" s="21"/>
     </row>
@@ -15360,7 +15358,7 @@
         <v>892</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>1105</v>
+        <v>1070</v>
       </c>
       <c r="H55" s="16"/>
     </row>
@@ -15384,7 +15382,7 @@
         <v>893</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>1106</v>
+        <v>1071</v>
       </c>
       <c r="H56" s="21"/>
     </row>
@@ -15486,7 +15484,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1059</v>
+        <v>1024</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -15510,7 +15508,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1060</v>
+        <v>1025</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -15534,7 +15532,7 @@
         <v>892</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1061</v>
+        <v>1026</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -16058,7 +16056,7 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1062</v>
+        <v>1027</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -16082,7 +16080,7 @@
         <v>892</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1063</v>
+        <v>1028</v>
       </c>
       <c r="H4" s="21"/>
     </row>
@@ -16106,7 +16104,7 @@
         <v>893</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1064</v>
+        <v>1029</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -16130,7 +16128,7 @@
         <v>893</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>1065</v>
+        <v>1030</v>
       </c>
       <c r="H6" s="21"/>
     </row>
@@ -16168,7 +16166,7 @@
         <v>892</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>1066</v>
+        <v>1031</v>
       </c>
       <c r="H8" s="16"/>
     </row>
@@ -16192,7 +16190,7 @@
         <v>892</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>1067</v>
+        <v>1032</v>
       </c>
       <c r="H9" s="21"/>
     </row>
@@ -16216,7 +16214,7 @@
         <v>892</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1068</v>
+        <v>1033</v>
       </c>
       <c r="H10" s="16"/>
     </row>
@@ -16240,7 +16238,7 @@
         <v>893</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>1069</v>
+        <v>1034</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -16322,7 +16320,7 @@
         <v>893</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1070</v>
+        <v>1035</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -16360,7 +16358,7 @@
         <v>893</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1071</v>
+        <v>1036</v>
       </c>
       <c r="H17" s="16"/>
     </row>

</xml_diff>

<commit_message>
Docs: Update the progression of the ASVS File
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\IdeaProjects\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867FC1B3-C43B-4388-AAE0-8BA869250391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E66F702-9CD3-4C1B-B48A-D3E6C39BDE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2298" uniqueCount="1133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2298" uniqueCount="1134">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -3464,6 +3464,9 @@
   </si>
   <si>
     <t>Users can review and revoke active sessions and granted consents via the Keycloak account management console (/realms/arcadehaven/account). The ArcadeHaven logout endpoint also triggers full session revocation via Keycloak.</t>
+  </si>
+  <si>
+    <t>Compliant</t>
   </si>
 </sst>
 </file>
@@ -3991,31 +3994,31 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.375</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.30769230769230771</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -4024,10 +4027,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="15" formatCode="General">
                   <c:v>0</c:v>
@@ -4169,7 +4172,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>5.2631578947368418E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -4178,28 +4181,28 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.125</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>4.5454545454545456E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.63636363636363635</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -4208,13 +4211,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>0.14285714285714285</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>0.3125</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -4383,7 +4386,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -4395,10 +4398,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>0.125</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4534,37 +4537,37 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>3.3333333333333333E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>9.6774193548387094E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.125</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>7.6923076923076927E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.10638297872340426</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.23076923076923078</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.5714285714285714</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.16666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -4573,13 +4576,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>0.15384615384615385</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>0.2857142857142857</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>0.35294117647058826</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -5214,11 +5217,11 @@
       </c>
       <c r="G6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" s="5">
         <f t="shared" ref="H6:H22" si="1">IF(F6=0,"",G6/F6)</f>
-        <v>0</v>
+        <v>5.2631578947368418E-2</v>
       </c>
       <c r="I6" s="4">
         <v>3</v>
@@ -5233,11 +5236,11 @@
       </c>
       <c r="L6" s="4">
         <f>COUNTIF('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" s="5">
         <f t="shared" ref="M6:M22" si="3">IF(B6=0,"",L6/B6)</f>
-        <v>0</v>
+        <v>3.3333333333333333E-2</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5301,11 +5304,11 @@
       </c>
       <c r="D8" s="4">
         <f>COUNTIFS('V3 - Web Frontend Security'!$F$2:$F$39,"Compliant",'V3 - Web Frontend Security'!$E$2:$E$39,1)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E8" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="F8" s="4">
         <v>11</v>
@@ -5331,11 +5334,11 @@
       </c>
       <c r="L8" s="4">
         <f>COUNTIF('V3 - Web Frontend Security'!$F$2:$F$39,"Compliant")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M8" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>9.6774193548387094E-2</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5350,22 +5353,22 @@
       </c>
       <c r="D9" s="7">
         <f>COUNTIFS('V4 - API and Web Service'!$F$2:$F$21,"Compliant",'V4 - API and Web Service'!$E$2:$E$21,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F9" s="7">
         <v>8</v>
       </c>
       <c r="G9" s="7">
         <f>COUNTIFS('V4 - API and Web Service'!$F$2:$F$21,"Compliant",'V4 - API and Web Service'!$E$2:$E$21,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I9" s="7">
         <v>6</v>
@@ -5380,11 +5383,11 @@
       </c>
       <c r="L9" s="7">
         <f>COUNTIF('V4 - API and Web Service'!$F$2:$F$21,"Compliant")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M9" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5399,11 +5402,11 @@
       </c>
       <c r="D10" s="4">
         <f>COUNTIFS('V5 - File Handling'!$F$2:$F$18,"Compliant",'V5 - File Handling'!$E$2:$E$18,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F10" s="4">
         <v>5</v>
@@ -5429,11 +5432,11 @@
       </c>
       <c r="L10" s="4">
         <f>COUNTIF('V5 - File Handling'!$F$2:$F$18,"Compliant")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7.6923076923076927E-2</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5448,22 +5451,22 @@
       </c>
       <c r="D11" s="7">
         <f>COUNTIFS('V6 - Authentication'!$F$2:$F$56,"Compliant",'V6 - Authentication'!$E$2:$E$56,1)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E11" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.30769230769230771</v>
       </c>
       <c r="F11" s="7">
         <v>22</v>
       </c>
       <c r="G11" s="7">
         <f>COUNTIFS('V6 - Authentication'!$F$2:$F$56,"Compliant",'V6 - Authentication'!$E$2:$E$56,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.5454545454545456E-2</v>
       </c>
       <c r="I11" s="7">
         <v>12</v>
@@ -5478,11 +5481,11 @@
       </c>
       <c r="L11" s="7">
         <f>COUNTIF('V6 - Authentication'!$F$2:$F$56,"Compliant")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M11" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.10638297872340426</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5546,22 +5549,22 @@
       </c>
       <c r="D13" s="7">
         <f>COUNTIFS('V8 - Authorization'!$F$2:$F$18,"Compliant",'V8 - Authorization'!$E$2:$E$18,1)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E13" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F13" s="7">
         <v>3</v>
       </c>
       <c r="G13" s="7">
         <f>COUNTIFS('V8 - Authorization'!$F$2:$F$18,"Compliant",'V8 - Authorization'!$E$2:$E$18,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="I13" s="7">
         <v>6</v>
@@ -5576,11 +5579,11 @@
       </c>
       <c r="L13" s="7">
         <f>COUNTIF('V8 - Authorization'!$F$2:$F$18,"Compliant")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M13" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.23076923076923078</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5595,11 +5598,11 @@
       </c>
       <c r="D14" s="4">
         <f>COUNTIFS('V9 - Self-contained Tokens'!$F$2:$F$10,"Compliant",'V9 - Self-contained Tokens'!$E$2:$E$10,1)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E14" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="4">
         <v>3</v>
@@ -5623,11 +5626,11 @@
       </c>
       <c r="L14" s="4">
         <f>COUNTIF('V9 - Self-contained Tokens'!$F$2:$F$10,"Compliant")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M14" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5653,11 +5656,11 @@
       </c>
       <c r="G15" s="7">
         <f>COUNTIFS('V10 - OAuth and OIDC'!$F$2:$F$44,"Compliant",'V10 - OAuth and OIDC'!$E$2:$E$44,2)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H15" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I15" s="7">
         <v>7</v>
@@ -5672,11 +5675,11 @@
       </c>
       <c r="L15" s="7">
         <f>COUNTIF('V10 - OAuth and OIDC'!$F$2:$F$44,"Compliant")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M15" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5691,41 +5694,41 @@
       </c>
       <c r="D16" s="4">
         <f>COUNTIFS('V11 - Cryptography'!$F$2:$F$32,"Compliant",'V11 - Cryptography'!$E$2:$E$32,1)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E16" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="4">
         <v>11</v>
       </c>
       <c r="G16" s="4">
         <f>COUNTIFS('V11 - Cryptography'!$F$2:$F$32,"Compliant",'V11 - Cryptography'!$E$2:$E$32,2)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H16" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.63636363636363635</v>
       </c>
       <c r="I16" s="4">
         <v>10</v>
       </c>
       <c r="J16" s="4">
         <f>COUNTIFS('V11 - Cryptography'!$F$2:$F$32,"Compliant",'V11 - Cryptography'!$E$2:$E$32,3)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K16" s="5">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="L16" s="4">
         <f>COUNTIF('V11 - Cryptography'!$F$2:$F$32,"Compliant")</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M16" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5838,22 +5841,22 @@
       </c>
       <c r="D19" s="7">
         <f>COUNTIFS('V14 - Data Protection'!$F$2:$F$17,"Compliant",'V14 - Data Protection'!$E$2:$E$17,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F19" s="7">
         <v>7</v>
       </c>
       <c r="G19" s="7">
         <f>COUNTIFS('V14 - Data Protection'!$F$2:$F$17,"Compliant",'V14 - Data Protection'!$E$2:$E$17,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="I19" s="7">
         <v>4</v>
@@ -5868,11 +5871,11 @@
       </c>
       <c r="L19" s="7">
         <f>COUNTIF('V14 - Data Protection'!$F$2:$F$17,"Compliant")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M19" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.15384615384615385</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5887,41 +5890,41 @@
       </c>
       <c r="D20" s="4">
         <f>COUNTIFS('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant",'V15 - Secure Coding and Archite'!$E$2:$E$26,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="F20" s="4">
         <v>10</v>
       </c>
       <c r="G20" s="4">
         <f>COUNTIFS('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant",'V15 - Secure Coding and Archite'!$E$2:$E$26,2)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H20" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I20" s="4">
         <v>8</v>
       </c>
       <c r="J20" s="4">
         <f>COUNTIFS('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant",'V15 - Secure Coding and Archite'!$E$2:$E$26,3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" s="5">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="L20" s="4">
         <f>COUNTIF('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M20" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5945,30 +5948,30 @@
       </c>
       <c r="G21" s="7">
         <f>COUNTIFS('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant",'V16 - Security Logging and Erro'!$E$2:$E$23,2)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H21" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.3125</v>
       </c>
       <c r="I21" s="7">
         <v>1</v>
       </c>
       <c r="J21" s="7">
         <f>COUNTIFS('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant",'V16 - Security Logging and Erro'!$E$2:$E$23,3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" s="8">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="7">
         <f>COUNTIF('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M21" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.35294117647058826</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6032,11 +6035,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>0</v>
+        <v>0.31773504273504272</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -6044,11 +6047,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>0</v>
+        <v>0.13518471982094274</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -6056,19 +6059,19 @@
       </c>
       <c r="J23" s="10">
         <f>SUM(J6:J22)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K23" s="11">
         <f>IFERROR(AVERAGE(K6:K22),"")</f>
-        <v>0</v>
+        <v>8.2812499999999997E-2</v>
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0</v>
+        <v>0.15881056867198226</v>
       </c>
     </row>
   </sheetData>
@@ -6203,7 +6206,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G3" s="16" t="s">
         <v>920</v>
@@ -6227,7 +6230,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G4" s="21" t="s">
         <v>921</v>
@@ -6251,7 +6254,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G5" s="16" t="s">
         <v>924</v>
@@ -6289,7 +6292,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G7" s="16" t="s">
         <v>925</v>
@@ -6463,7 +6466,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G3" s="16" t="s">
         <v>1098</v>
@@ -6487,7 +6490,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G4" s="21" t="s">
         <v>1099</v>
@@ -6633,7 +6636,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G11" s="21" t="s">
         <v>1103</v>
@@ -6657,7 +6660,7 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G12" s="16" t="s">
         <v>1104</v>
@@ -7165,7 +7168,7 @@
         <v>2</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G34" s="21" t="s">
         <v>1123</v>
@@ -7189,7 +7192,7 @@
         <v>2</v>
       </c>
       <c r="F35" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G35" s="16" t="s">
         <v>1125</v>
@@ -7404,7 +7407,7 @@
       <formula>"Not Applicable"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="F2:F1044" xr:uid="{00000000-0002-0000-0A00-000000000000}">
       <formula1>"Not Started,In Progress,Compliant,Not Applicable"</formula1>
       <formula2>0</formula2>
@@ -7593,7 +7596,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G8" s="16" t="s">
         <v>939</v>
@@ -7641,7 +7644,7 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>941</v>
@@ -7665,7 +7668,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G11" s="21" t="s">
         <v>942</v>
@@ -7727,7 +7730,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G14" s="16" t="s">
         <v>944</v>
@@ -7751,7 +7754,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G15" s="21" t="s">
         <v>945</v>
@@ -7775,7 +7778,7 @@
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G16" s="16" t="s">
         <v>946</v>
@@ -7859,7 +7862,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G20" s="27" t="s">
         <v>948</v>
@@ -7883,7 +7886,7 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G21" s="27" t="s">
         <v>949</v>
@@ -7907,7 +7910,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G22" s="27" t="s">
         <v>950</v>
@@ -7931,7 +7934,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G23" s="21" t="s">
         <v>951</v>
@@ -7993,7 +7996,7 @@
         <v>3</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G26" s="21" t="s">
         <v>953</v>
@@ -8031,7 +8034,7 @@
         <v>2</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G28" s="16" t="s">
         <v>954</v>
@@ -9259,7 +9262,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G6" s="16" t="s">
         <v>913</v>
@@ -9307,7 +9310,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G8" s="16" t="s">
         <v>914</v>
@@ -9763,7 +9766,7 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G10" s="21" t="s">
         <v>962</v>
@@ -9833,7 +9836,7 @@
         <v>3</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>964</v>
@@ -9871,7 +9874,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G15" s="16" t="s">
         <v>965</v>
@@ -9919,7 +9922,7 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G17" s="16" t="s">
         <v>967</v>
@@ -9967,7 +9970,7 @@
         <v>2</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G19" s="16" t="s">
         <v>969</v>
@@ -10015,7 +10018,7 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>971</v>
@@ -10281,7 +10284,7 @@
         <v>2</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G6" s="21" t="s">
         <v>976</v>
@@ -10305,7 +10308,7 @@
         <v>2</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G7" s="16" t="s">
         <v>975</v>
@@ -10415,7 +10418,7 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G12" s="21" t="s">
         <v>972</v>
@@ -10587,7 +10590,7 @@
         <v>2</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G20" s="16" t="s">
         <v>982</v>
@@ -10635,7 +10638,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G22" s="16" t="s">
         <v>984</v>
@@ -10659,7 +10662,7 @@
         <v>3</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G23" s="21" t="s">
         <v>985</v>
@@ -11155,7 +11158,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G3" s="29" t="s">
         <v>1000</v>
@@ -12855,7 +12858,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G24" s="25" t="s">
         <v>1014</v>
@@ -12879,7 +12882,7 @@
         <v>1</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G25" s="26" t="s">
         <v>1015</v>
@@ -12903,7 +12906,7 @@
         <v>1</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G26" s="25" t="s">
         <v>1016</v>
@@ -13291,7 +13294,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G3" s="16" t="s">
         <v>1022</v>
@@ -13421,7 +13424,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G9" s="16" t="s">
         <v>910</v>
@@ -13821,7 +13824,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G5" s="16" t="s">
         <v>928</v>
@@ -14455,7 +14458,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G14" s="21" t="s">
         <v>1047</v>
@@ -14589,7 +14592,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G20" s="16" t="s">
         <v>1052</v>
@@ -14613,7 +14616,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G21" s="21" t="s">
         <v>1053</v>
@@ -14811,7 +14814,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G30" s="21" t="s">
         <v>1057</v>
@@ -15331,7 +15334,7 @@
         <v>2</v>
       </c>
       <c r="F54" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G54" s="21" t="s">
         <v>1069</v>
@@ -15398,7 +15401,7 @@
       <formula>"Not Applicable"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="F2:F1056" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Not Started,In Progress,Compliant,Not Applicable"</formula1>
       <formula2>0</formula2>
@@ -16163,7 +16166,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G8" s="16" t="s">
         <v>1031</v>
@@ -16187,7 +16190,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G9" s="21" t="s">
         <v>1032</v>
@@ -16211,7 +16214,7 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>892</v>
+        <v>1133</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>1033</v>

</xml_diff>

<commit_message>
Docs: Update the ASVS file #3
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\IdeaProjects\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E66F702-9CD3-4C1B-B48A-D3E6C39BDE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4419B5-B5BB-4926-B095-967C16B198F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2298" uniqueCount="1134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2310" uniqueCount="1146">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -3467,6 +3467,42 @@
   </si>
   <si>
     <t>Compliant</t>
+  </si>
+  <si>
+    <t>The entire data access layer uses Spring Data JPA with typed repositories</t>
+  </si>
+  <si>
+    <t>ArcadeHaven does not use SpEL with user input. The @PreAuthorize annotations use SpEL with static expressions (“hasRole(‘ADMIN’)”)</t>
+  </si>
+  <si>
+    <t>Logging uses only SLF4J with parameterized placeholders (log.warn(“message: {}”, value))</t>
+  </si>
+  <si>
+    <t>All request DTOs use Bean Validation</t>
+  </si>
+  <si>
+    <t>All validation is performed server-side using Spring Bean Validation in the controller/service layer. There is no frontend implementation that performs client-side validation, so there is no risk of bypass. The tracker must be updated.</t>
+  </si>
+  <si>
+    <t>The Order uses a state machine (OrderStatus: PENDING → COMPLETED), and the Order.complete() method validates that the status is PENDING before transitioning. The LibraryEntry is only created after the Order is COMPLETED. The game follows the PENDING → APPROVED/REJECTED flow with validation in the AdminService. The tracker must be updated.</t>
+  </si>
+  <si>
+    <t>JWT validation is performed exclusively on the server by the Spring Security JWT decoder, using Keycloak's JWKS endpoint. No tokens are validated on the client side or via frontend logic. The tracker must be updated.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven uses dynamic JWTs issued by Keycloak with exp and iat claims. There are no static API keys for user authentication. The Keycloak Admin Client uses a service account with the client credentials flow—credentials configured via environment variables, not hardcoded. The tracker needs to be updated.</t>
+  </si>
+  <si>
+    <t>Keycloak issues a new JWT access token and refresh token with each successful authentication. Logging out via a POST request to /api/auth/logout revokes all active tokens. Spring Boot does not maintain session state (stateless JWT). The tracker must be updated.</t>
+  </si>
+  <si>
+    <t>POST /api/auth/logout revokes all of the user's active sessions in Keycloak via UserResource.logout() (Keycloak Admin Client). Tokens naturally expire based on the exp claim. The tracker is out of date, this check should be marked as “Compliant” (matches V6.8.3 / V10.4.9, which have already been implemented).</t>
+  </si>
+  <si>
+    <t>The authentication flow requires explicit user action (submitting credentials to Keycloak). Spring Boot does not automatically create sessions, it is stateless. The JWT is only issued after successful authentication. The tracker must be updated.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> All authorization is server-side: SecurityConfig with rules based on path/role, @PreAuthorize(“hasRole(...)”)</t>
   </si>
 </sst>
 </file>
@@ -3988,10 +4024,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0.375</c:v>
@@ -4006,10 +4042,10 @@
                   <c:v>0.30769230769230771</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.5</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>1</c:v>
@@ -4172,7 +4208,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>5.2631578947368418E-2</c:v>
+                  <c:v>0.10526315789473684</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -4190,7 +4226,7 @@
                   <c:v>4.5454545454545456E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>8.3333333333333329E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.33333333333333331</c:v>
@@ -4537,10 +4573,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>3.3333333333333333E-2</c:v>
+                  <c:v>0.13333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.23076923076923078</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>9.6774193548387094E-2</c:v>
@@ -4555,10 +4591,10 @@
                   <c:v>0.10638297872340426</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>0.26315789473684209</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.23076923076923078</c:v>
+                  <c:v>0.30769230769230771</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0.5714285714285714</c:v>
@@ -5206,22 +5242,22 @@
       </c>
       <c r="D6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,1)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" s="5">
         <f t="shared" ref="E6:E20" si="0">IF(C6=0,"",D6/C6)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F6" s="4">
         <v>19</v>
       </c>
       <c r="G6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,2)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6" s="5">
         <f t="shared" ref="H6:H22" si="1">IF(F6=0,"",G6/F6)</f>
-        <v>5.2631578947368418E-2</v>
+        <v>0.10526315789473684</v>
       </c>
       <c r="I6" s="4">
         <v>3</v>
@@ -5236,11 +5272,11 @@
       </c>
       <c r="L6" s="4">
         <f>COUNTIF('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M6" s="5">
         <f t="shared" ref="M6:M22" si="3">IF(B6=0,"",L6/B6)</f>
-        <v>3.3333333333333333E-2</v>
+        <v>0.13333333333333333</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5255,11 +5291,11 @@
       </c>
       <c r="D7" s="7">
         <f>COUNTIFS('V2 - Validation and Business Lo'!$F$2:$F$18,"Compliant",'V2 - Validation and Business Lo'!$E$2:$E$18,1)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E7" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="F7" s="7">
         <v>7</v>
@@ -5285,11 +5321,11 @@
       </c>
       <c r="L7" s="7">
         <f>COUNTIF('V2 - Validation and Business Lo'!$F$2:$F$18,"Compliant")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M7" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.23076923076923078</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5500,22 +5536,22 @@
       </c>
       <c r="D12" s="4">
         <f>COUNTIFS('V7 - Session Management'!$F$2:$F$26,"Compliant",'V7 - Session Management'!$E$2:$E$26,1)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E12" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="F12" s="4">
         <v>12</v>
       </c>
       <c r="G12" s="4">
         <f>COUNTIFS('V7 - Session Management'!$F$2:$F$26,"Compliant",'V7 - Session Management'!$E$2:$E$26,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="I12" s="4">
         <v>1</v>
@@ -5530,11 +5566,11 @@
       </c>
       <c r="L12" s="4">
         <f>COUNTIF('V7 - Session Management'!$F$2:$F$26,"Compliant")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M12" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.26315789473684209</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5549,11 +5585,11 @@
       </c>
       <c r="D13" s="7">
         <f>COUNTIFS('V8 - Authorization'!$F$2:$F$18,"Compliant",'V8 - Authorization'!$E$2:$E$18,1)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" s="8">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="F13" s="7">
         <v>3</v>
@@ -5579,11 +5615,11 @@
       </c>
       <c r="L13" s="7">
         <f>COUNTIF('V8 - Authorization'!$F$2:$F$18,"Compliant")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" s="8">
         <f t="shared" si="3"/>
-        <v>0.23076923076923078</v>
+        <v>0.30769230769230771</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6035,11 +6071,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>0.31773504273504272</v>
+        <v>0.44551282051282048</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -6047,11 +6083,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>0.13518471982094274</v>
+        <v>0.1431826558374546</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -6067,11 +6103,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0.15881056867198226</v>
+        <v>0.19827234528546164</v>
       </c>
     </row>
   </sheetData>
@@ -9015,7 +9051,7 @@
       </c>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>720</v>
       </c>
@@ -11266,7 +11302,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G8" s="29"/>
       <c r="H8" s="16"/>
@@ -11288,9 +11324,11 @@
         <v>1</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="30"/>
+        <v>1133</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>1134</v>
+      </c>
       <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11490,9 +11528,11 @@
         <v>1</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="G18" s="30"/>
+        <v>1133</v>
+      </c>
+      <c r="G18" s="30" t="s">
+        <v>1135</v>
+      </c>
       <c r="H18" s="21"/>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11604,7 +11644,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="28" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G23" s="29"/>
       <c r="H23" s="16"/>
@@ -11674,9 +11714,11 @@
         <v>2</v>
       </c>
       <c r="F26" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="G26" s="30"/>
+        <v>1133</v>
+      </c>
+      <c r="G26" s="30" t="s">
+        <v>1136</v>
+      </c>
       <c r="H26" s="21"/>
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11802,7 +11844,7 @@
         <v>2</v>
       </c>
       <c r="F32" s="28" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G32" s="29"/>
       <c r="H32" s="16"/>
@@ -11838,7 +11880,7 @@
         <v>1</v>
       </c>
       <c r="F34" s="28" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G34" s="29"/>
       <c r="H34" s="16"/>
@@ -12068,12 +12110,14 @@
         <v>1</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="29"/>
+        <v>1133</v>
+      </c>
+      <c r="G7" s="29" t="s">
+        <v>1137</v>
+      </c>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>120</v>
       </c>
@@ -12090,9 +12134,11 @@
         <v>1</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="30"/>
+        <v>1133</v>
+      </c>
+      <c r="G8" s="30" t="s">
+        <v>1138</v>
+      </c>
       <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -12131,7 +12177,7 @@
       <c r="G10" s="31"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>128</v>
       </c>
@@ -12148,9 +12194,11 @@
         <v>1</v>
       </c>
       <c r="F11" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="29"/>
+        <v>1133</v>
+      </c>
+      <c r="G11" s="29" t="s">
+        <v>1139</v>
+      </c>
       <c r="H11" s="16"/>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -12700,7 +12748,7 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G17" s="25" t="s">
         <v>1008</v>
@@ -13124,7 +13172,7 @@
         <v>2</v>
       </c>
       <c r="F36" s="18" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G36" s="26"/>
       <c r="H36" s="21"/>
@@ -15553,7 +15601,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>414</v>
       </c>
@@ -15570,12 +15618,14 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="16"/>
+        <v>1133</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>1140</v>
+      </c>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>414</v>
       </c>
@@ -15592,9 +15642,11 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="21"/>
+        <v>1133</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>1141</v>
+      </c>
       <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15614,12 +15666,12 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>414</v>
       </c>
@@ -15636,9 +15688,11 @@
         <v>1</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G10" s="21"/>
+        <v>1133</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>1142</v>
+      </c>
       <c r="H10" s="21"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -15713,7 +15767,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>430</v>
       </c>
@@ -15730,9 +15784,11 @@
         <v>1</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" s="16"/>
+        <v>1133</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>1143</v>
+      </c>
       <c r="H15" s="16"/>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15796,7 +15852,7 @@
         <v>2</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
@@ -15939,7 +15995,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>450</v>
       </c>
@@ -15956,9 +16012,11 @@
         <v>2</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G26" s="21"/>
+        <v>1133</v>
+      </c>
+      <c r="G26" s="21" t="s">
+        <v>1144</v>
+      </c>
       <c r="H26" s="21"/>
     </row>
   </sheetData>
@@ -16259,7 +16317,7 @@
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>476</v>
       </c>
@@ -16276,9 +16334,11 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="16"/>
+        <v>1133</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>1145</v>
+      </c>
       <c r="H13" s="16"/>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Docs: Placeholder of the references on the ASVS file #3
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\IdeaProjects\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4419B5-B5BB-4926-B095-967C16B198F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FAC981-2A62-47A0-B4F7-4C0A4CF732DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2310" uniqueCount="1146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="1197">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -3503,6 +3503,159 @@
   </si>
   <si>
     <t xml:space="preserve"> All authorization is server-side: SecurityConfig with rules based on path/role, @PreAuthorize(“hasRole(...)”)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Dto/Request/RegisterRequest.java; Api/src/main/.../Validation/NoHtmlValidator.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java; Controller/AuthController.java; Controller/OrderController.java; Controller/PublisherController.java; Controller/AdminController.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Controller/OrderController.java; Controller/PublisherController.java; Controller/AdminController.java; Controller/GameController.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Controller/LibraryController.java; Controller/OrderController.java</t>
+  </si>
+  <si>
+    <t>Api/pom.xml (spring-boot-starter-web -&gt; embedded Tomcat)</t>
+  </si>
+  <si>
+    <t>Api/src/main/resources/application.properties (max-file-size=25MB); Exception/GlobalExceptionHandler.java (HTTP 413)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Service/AuthService.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/RateLimitFilter.java (Bucket4j, 20 req/min per IP)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Config/AdminInitializer.java (env vars ADMIN_USERNAME/ADMIN_PASSWORD)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Dto/Request/RegisterRequest.java (no secret-question field)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java; Api/src/main/resources/application.properties (jwk-set-uri)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java; Controller/AdminController.java; Controller/PublisherController.java; Controller/OrderController.java; Security/KeycloakRoleConverter.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Service/GameService.java (findByIdAndPublisher); Service/OrderService.java; Service/LibraryService.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Dto/Response/UserResponse.java; Dto/Response/OrderResponse.java; Dto/Response/GameResponse.java; Dto/Response/LibraryEntryResponse.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (Spring Security JWT decoder)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (Nimbus JOSE, RS256 only)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java; application.properties (jwk-set-uri)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (Spring Security validates exp/nbf)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java; Service/AuthService.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (iss/aud validation); Keycloak PKCE/state/nonce</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/KeycloakRoleConverter.java; Security/SecurityConfig.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/KeycloakRoleConverter.java (sub=UUID); Security/SecurityConfig.java (iss)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/KeycloakRoleConverter.java (sub UUID, non-reassignable)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java; application.properties (issuer-uri)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Service/PasswordPolicyService.java; Security/SecurityConfig.java; Api/pom.xml</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (RS256/HS256, BCrypt&gt;=12, TLS1.2+)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (BCryptPasswordEncoder.matches, Nimbus JOSE)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (TLS1.2+ only, no ECB)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (TLS AES-GCM cipher suites)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (HMAC-SHA256 JWT integrity)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Service/PasswordPolicyService.java (SHA-1 HIBP-only, non-cryptographic)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Service/AuthService.java (Keycloak BCrypt &gt;= work factor 12)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java (HMAC-SHA256 256-bit / RS256)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Service/AuthService.java (Keycloak BCrypt adaptive cost)</t>
+  </si>
+  <si>
+    <t>Java SecureRandom (NativePRNGNonBlocking on Linux, JVM built-in)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java; application.properties (jwt.*)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Controller/AuthController.java; Dto/Request/RegisterRequest.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Service/PasswordPolicyService.java (HIBP 5-char prefix only)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/RateLimitFilter.java; Exception/GlobalExceptionHandler.java; application.properties</t>
+  </si>
+  <si>
+    <t>Api/docker-compose.yml (separate containers, network isolation)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Dto/Response/UserResponse.java; Dto/Response/GameResponse.java; Dto/Response/OrderResponse.java; Dto/Response/LibraryEntryResponse.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Dto/Request/RegisterRequest.java; Dto/Request/CreateGameRequest.java; Dto/Request/UpdateProfileRequest.java; Dto/Request/AddOrderItemRequest.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Dto/Request/ (all request DTOs — Java static typing + Bean Validation)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityConfig.java; all controllers (@RequestParam/@RequestBody separate binding)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityAuditService.java (Instant.now() UTC); Security/SecurityEventHandler.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityAuditService.java (SECURITY_AUDIT logger, stdout + logs/arcadehaven.log)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Security/SecurityAuditService.java (recordAccessDenied); Security/SecurityEventHandler.java</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Exception/GlobalExceptionHandler.java (generic error messages, no stack traces)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Exception/GlobalExceptionHandler.java; Security/SecurityConfig.java (deny-all default)</t>
+  </si>
+  <si>
+    <t>Api/src/main/.../Exception/GlobalExceptionHandler.java (@ExceptionHandler(Exception.class) catch-all)</t>
   </si>
 </sst>
 </file>
@@ -6247,7 +6400,9 @@
       <c r="G3" s="16" t="s">
         <v>920</v>
       </c>
-      <c r="H3" s="16"/>
+      <c r="H3" s="16" t="s">
+        <v>1161</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -6271,7 +6426,9 @@
       <c r="G4" s="21" t="s">
         <v>921</v>
       </c>
-      <c r="H4" s="21"/>
+      <c r="H4" s="21" t="s">
+        <v>1162</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
@@ -6295,7 +6452,9 @@
       <c r="G5" s="16" t="s">
         <v>924</v>
       </c>
-      <c r="H5" s="16"/>
+      <c r="H5" s="16" t="s">
+        <v>1163</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
@@ -6333,7 +6492,9 @@
       <c r="G7" s="16" t="s">
         <v>925</v>
       </c>
-      <c r="H7" s="16"/>
+      <c r="H7" s="16" t="s">
+        <v>1164</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
@@ -6507,7 +6668,9 @@
       <c r="G3" s="16" t="s">
         <v>1098</v>
       </c>
-      <c r="H3" s="16"/>
+      <c r="H3" s="16" t="s">
+        <v>1165</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -6531,7 +6694,9 @@
       <c r="G4" s="21" t="s">
         <v>1099</v>
       </c>
-      <c r="H4" s="21"/>
+      <c r="H4" s="21" t="s">
+        <v>1166</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
@@ -6677,7 +6842,9 @@
       <c r="G11" s="21" t="s">
         <v>1103</v>
       </c>
-      <c r="H11" s="21"/>
+      <c r="H11" s="21" t="s">
+        <v>1167</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
@@ -6701,7 +6868,9 @@
       <c r="G12" s="16" t="s">
         <v>1104</v>
       </c>
-      <c r="H12" s="16"/>
+      <c r="H12" s="16" t="s">
+        <v>1168</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="73.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
@@ -7209,7 +7378,9 @@
       <c r="G34" s="21" t="s">
         <v>1123</v>
       </c>
-      <c r="H34" s="21"/>
+      <c r="H34" s="21" t="s">
+        <v>1169</v>
+      </c>
     </row>
     <row r="35" spans="1:8" ht="120" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
@@ -7233,7 +7404,9 @@
       <c r="G35" s="16" t="s">
         <v>1125</v>
       </c>
-      <c r="H35" s="16"/>
+      <c r="H35" s="16" t="s">
+        <v>1170</v>
+      </c>
     </row>
     <row r="36" spans="1:8" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
@@ -7637,7 +7810,9 @@
       <c r="G8" s="16" t="s">
         <v>939</v>
       </c>
-      <c r="H8" s="16"/>
+      <c r="H8" s="16" t="s">
+        <v>1171</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="225" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
@@ -7685,7 +7860,9 @@
       <c r="G10" s="16" t="s">
         <v>941</v>
       </c>
-      <c r="H10" s="16"/>
+      <c r="H10" s="16" t="s">
+        <v>1172</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="240" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
@@ -7709,7 +7886,9 @@
       <c r="G11" s="21" t="s">
         <v>942</v>
       </c>
-      <c r="H11" s="21"/>
+      <c r="H11" s="21" t="s">
+        <v>1173</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="195" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
@@ -7771,7 +7950,9 @@
       <c r="G14" s="16" t="s">
         <v>944</v>
       </c>
-      <c r="H14" s="16"/>
+      <c r="H14" s="16" t="s">
+        <v>1174</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
@@ -7795,7 +7976,9 @@
       <c r="G15" s="21" t="s">
         <v>945</v>
       </c>
-      <c r="H15" s="21"/>
+      <c r="H15" s="21" t="s">
+        <v>1175</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
@@ -7819,7 +8002,9 @@
       <c r="G16" s="16" t="s">
         <v>946</v>
       </c>
-      <c r="H16" s="16"/>
+      <c r="H16" s="16" t="s">
+        <v>1176</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
@@ -7903,7 +8088,9 @@
       <c r="G20" s="27" t="s">
         <v>948</v>
       </c>
-      <c r="H20" s="16"/>
+      <c r="H20" s="16" t="s">
+        <v>1177</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="195" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
@@ -7927,7 +8114,9 @@
       <c r="G21" s="27" t="s">
         <v>949</v>
       </c>
-      <c r="H21" s="21"/>
+      <c r="H21" s="21" t="s">
+        <v>1178</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="180" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
@@ -7951,7 +8140,9 @@
       <c r="G22" s="27" t="s">
         <v>950</v>
       </c>
-      <c r="H22" s="16"/>
+      <c r="H22" s="16" t="s">
+        <v>1179</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="180" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
@@ -7975,7 +8166,9 @@
       <c r="G23" s="21" t="s">
         <v>951</v>
       </c>
-      <c r="H23" s="21"/>
+      <c r="H23" s="21" t="s">
+        <v>1180</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
@@ -8037,7 +8230,9 @@
       <c r="G26" s="21" t="s">
         <v>953</v>
       </c>
-      <c r="H26" s="21"/>
+      <c r="H26" s="21" t="s">
+        <v>1181</v>
+      </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
@@ -8075,7 +8270,9 @@
       <c r="G28" s="16" t="s">
         <v>954</v>
       </c>
-      <c r="H28" s="16"/>
+      <c r="H28" s="16" t="s">
+        <v>1182</v>
+      </c>
     </row>
     <row r="29" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
@@ -9303,7 +9500,9 @@
       <c r="G6" s="16" t="s">
         <v>913</v>
       </c>
-      <c r="H6" s="16"/>
+      <c r="H6" s="16" t="s">
+        <v>1183</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="50.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
@@ -9351,7 +9550,9 @@
       <c r="G8" s="16" t="s">
         <v>914</v>
       </c>
-      <c r="H8" s="16"/>
+      <c r="H8" s="16" t="s">
+        <v>1184</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
@@ -9807,7 +10008,9 @@
       <c r="G10" s="21" t="s">
         <v>962</v>
       </c>
-      <c r="H10" s="21"/>
+      <c r="H10" s="21" t="s">
+        <v>1185</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
@@ -9877,7 +10080,9 @@
       <c r="G13" s="16" t="s">
         <v>964</v>
       </c>
-      <c r="H13" s="16"/>
+      <c r="H13" s="16" t="s">
+        <v>1186</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
@@ -9915,7 +10120,9 @@
       <c r="G15" s="16" t="s">
         <v>965</v>
       </c>
-      <c r="H15" s="16"/>
+      <c r="H15" s="16" t="s">
+        <v>1187</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="135" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
@@ -9963,7 +10170,9 @@
       <c r="G17" s="16" t="s">
         <v>967</v>
       </c>
-      <c r="H17" s="16"/>
+      <c r="H17" s="16" t="s">
+        <v>1188</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
@@ -10011,7 +10220,9 @@
       <c r="G19" s="16" t="s">
         <v>969</v>
       </c>
-      <c r="H19" s="16"/>
+      <c r="H19" s="16" t="s">
+        <v>1189</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
@@ -10059,7 +10270,9 @@
       <c r="G21" s="16" t="s">
         <v>971</v>
       </c>
-      <c r="H21" s="16"/>
+      <c r="H21" s="16" t="s">
+        <v>1190</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
@@ -10325,7 +10538,9 @@
       <c r="G6" s="21" t="s">
         <v>976</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="21" t="s">
+        <v>1191</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="135" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
@@ -10349,7 +10564,9 @@
       <c r="G7" s="16" t="s">
         <v>975</v>
       </c>
-      <c r="H7" s="16"/>
+      <c r="H7" s="16" t="s">
+        <v>1192</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
@@ -10459,7 +10676,9 @@
       <c r="G12" s="21" t="s">
         <v>972</v>
       </c>
-      <c r="H12" s="21"/>
+      <c r="H12" s="21" t="s">
+        <v>1193</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
@@ -10631,7 +10850,9 @@
       <c r="G20" s="16" t="s">
         <v>982</v>
       </c>
-      <c r="H20" s="16"/>
+      <c r="H20" s="16" t="s">
+        <v>1194</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="195" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
@@ -10679,7 +10900,9 @@
       <c r="G22" s="16" t="s">
         <v>984</v>
       </c>
-      <c r="H22" s="16"/>
+      <c r="H22" s="16" t="s">
+        <v>1195</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="225" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
@@ -10703,7 +10926,9 @@
       <c r="G23" s="21" t="s">
         <v>985</v>
       </c>
-      <c r="H23" s="21"/>
+      <c r="H23" s="21" t="s">
+        <v>1196</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F23">
@@ -11199,7 +11424,9 @@
       <c r="G3" s="29" t="s">
         <v>1000</v>
       </c>
-      <c r="H3" s="16"/>
+      <c r="H3" s="16" t="s">
+        <v>1146</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -12383,7 +12610,7 @@
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="81.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="115.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
@@ -12911,7 +13138,9 @@
       <c r="G24" s="25" t="s">
         <v>1014</v>
       </c>
-      <c r="H24" s="16"/>
+      <c r="H24" s="16" t="s">
+        <v>1147</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
@@ -12935,7 +13164,9 @@
       <c r="G25" s="26" t="s">
         <v>1015</v>
       </c>
-      <c r="H25" s="21"/>
+      <c r="H25" s="21" t="s">
+        <v>1148</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
@@ -12959,7 +13190,9 @@
       <c r="G26" s="25" t="s">
         <v>1016</v>
       </c>
-      <c r="H26" s="16"/>
+      <c r="H26" s="16" t="s">
+        <v>1149</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
@@ -13347,7 +13580,9 @@
       <c r="G3" s="16" t="s">
         <v>1022</v>
       </c>
-      <c r="H3" s="16"/>
+      <c r="H3" s="16" t="s">
+        <v>1150</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -13477,7 +13712,9 @@
       <c r="G9" s="16" t="s">
         <v>910</v>
       </c>
-      <c r="H9" s="16"/>
+      <c r="H9" s="16" t="s">
+        <v>1151</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
@@ -13877,7 +14114,9 @@
       <c r="G5" s="16" t="s">
         <v>928</v>
       </c>
-      <c r="H5" s="16"/>
+      <c r="H5" s="16" t="s">
+        <v>1152</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
@@ -14511,7 +14750,9 @@
       <c r="G14" s="21" t="s">
         <v>1047</v>
       </c>
-      <c r="H14" s="21"/>
+      <c r="H14" s="21" t="s">
+        <v>1153</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
@@ -14645,7 +14886,9 @@
       <c r="G20" s="16" t="s">
         <v>1052</v>
       </c>
-      <c r="H20" s="16"/>
+      <c r="H20" s="16" t="s">
+        <v>1154</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
@@ -14669,7 +14912,9 @@
       <c r="G21" s="21" t="s">
         <v>1053</v>
       </c>
-      <c r="H21" s="21"/>
+      <c r="H21" s="21" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
@@ -14867,7 +15112,9 @@
       <c r="G30" s="21" t="s">
         <v>1057</v>
       </c>
-      <c r="H30" s="21"/>
+      <c r="H30" s="21" t="s">
+        <v>1156</v>
+      </c>
     </row>
     <row r="31" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
@@ -15387,7 +15634,9 @@
       <c r="G54" s="21" t="s">
         <v>1069</v>
       </c>
-      <c r="H54" s="21"/>
+      <c r="H54" s="21" t="s">
+        <v>1157</v>
+      </c>
     </row>
     <row r="55" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
@@ -16229,7 +16478,9 @@
       <c r="G8" s="16" t="s">
         <v>1031</v>
       </c>
-      <c r="H8" s="16"/>
+      <c r="H8" s="16" t="s">
+        <v>1158</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
@@ -16253,7 +16504,9 @@
       <c r="G9" s="21" t="s">
         <v>1032</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="21" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
@@ -16277,7 +16530,9 @@
       <c r="G10" s="16" t="s">
         <v>1033</v>
       </c>
-      <c r="H10" s="16"/>
+      <c r="H10" s="16" t="s">
+        <v>1160</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">

</xml_diff>

<commit_message>
fix: AuthService due to test failure. update ASVS #3
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\IdeaProjects\desofs2026-wed_nap_2\Deliverables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\Desktop\DESOFS\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_04184BE8FAEDA34675B62AFB6F0CE81C351DD775" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7EA40A9-DFFB-4948-9161-EC9ABE4DF8D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -32,25 +32,12 @@
     <sheet name="V16 - Security Logging and Erro" sheetId="17" r:id="rId17"/>
     <sheet name="V17 - WebRTC" sheetId="18" r:id="rId18"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2446" uniqueCount="1282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2450" uniqueCount="1286">
   <si>
     <t>Section ID</t>
   </si>
@@ -3908,6 +3895,18 @@
   </si>
   <si>
     <t>No signaling server is used. Malformed signaling message handling is not applicable to the current project scope.</t>
+  </si>
+  <si>
+    <t>ArcadeHaven escapes special characters in inputs through th NoHtml validator</t>
+  </si>
+  <si>
+    <t>Api/src/main/java/…/Validation/NoHtmlValidator</t>
+  </si>
+  <si>
+    <t>ArcadeHaven domain classes apply range validation techniques to prevent overflow</t>
+  </si>
+  <si>
+    <t>Api/src/main/java/.../Service/Domain/Game Api/src/main/java/.../Service/Domain/OrderItem</t>
   </si>
 </sst>
 </file>
@@ -4614,7 +4613,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0.10526315789473684</c:v>
+                  <c:v>0.21052631578947367</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -4979,7 +4978,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0.13333333333333333</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.23076923076923078</c:v>
@@ -5656,11 +5655,11 @@
       </c>
       <c r="G6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,2)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H6" s="5">
         <f t="shared" ref="H6:H22" si="1">IF(F6=0,"",G6/F6)</f>
-        <v>0.10526315789473684</v>
+        <v>0.21052631578947367</v>
       </c>
       <c r="I6" s="4">
         <v>3</v>
@@ -5675,11 +5674,11 @@
       </c>
       <c r="L6" s="4">
         <f>COUNTIF('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M6" s="5">
         <f t="shared" ref="M6:M22" si="3">IF(B6=0,"",L6/B6)</f>
-        <v>0.13333333333333333</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6486,11 +6485,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>0.17259442054333696</v>
+        <v>0.17878637100773323</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -6506,11 +6505,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0.22441613613513484</v>
+        <v>0.22833770476258583</v>
       </c>
     </row>
   </sheetData>
@@ -12031,10 +12030,14 @@
         <v>2</v>
       </c>
       <c r="F14" s="28" t="s">
-        <v>115</v>
-      </c>
-      <c r="G14" s="29"/>
-      <c r="H14" s="16"/>
+        <v>12</v>
+      </c>
+      <c r="G14" s="29" t="s">
+        <v>1282</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>1283</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
@@ -12409,10 +12412,14 @@
         <v>2</v>
       </c>
       <c r="F31" s="28" t="s">
-        <v>115</v>
-      </c>
-      <c r="G31" s="30"/>
-      <c r="H31" s="21"/>
+        <v>12</v>
+      </c>
+      <c r="G31" s="30" t="s">
+        <v>1284</v>
+      </c>
+      <c r="H31" s="21" t="s">
+        <v>1285</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">

</xml_diff>

<commit_message>
feat: Improvement the API with the ASVS Rules specific about Authentication, Logs, RateLimit and Security Audit #9 #10 #12 #13 #16
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -453,7 +453,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -632,7 +632,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -809,7 +809,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -984,7 +984,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1159,7 +1159,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1210,7 +1210,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1240,7 +1240,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4847,17 +4847,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>ArcadeHaven's cryptographic operations are documented across RNF-01, RNF-02, RNF-05, and RNF-08: BCrypt (work factor 12) for password hashing, HMAC-SHA256 for JWT signing, TLS 1.2+ for transport, and CSPRNG for activation key generation. A consolidated cryptographic inventory — listing each operation with its algorithm parameters, key storage location, data types protected, and usage restrictions — is being assembled from these sources into a single reference document.</t>
+          <t>Cryptographic inventory documented in Documentation/CryptographicInventory.md. Covers 6 assets: KA-01 JWT RS256 (Keycloak, 2048-bit RSA), KA-02 BCrypt cost-12 (Keycloak password storage), KA-03 CSPRNG 128-bit SecureRandom (activation key generation), KA-04 SHA-1 HIBP k-anonymity (non-cryptographic, protocol-mandated), KA-05 TLS 1.2/1.3 AES-256-GCM ECDHE, KA-06 SSH RSA/ECDSA host key verification. Each asset includes algorithm justification, key size, usage, config location, and status. Prohibited algorithms table included (MD5, SHA-1 for crypto, DES/3DES, RC4, ECB, PKCS#1v1.5, alg:none).</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>Api/pom.xml (cyclonedx-maven-plugin 2.9.0); .github/workflows/build.yml (makeAggregateBom + SBOM artifact upload)</t>
+          <t>Documentation/CryptographicInventory.md (sections 1-2, 4-5)</t>
         </is>
       </c>
     </row>
@@ -5009,17 +5009,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
-          <t>ArcadeHaven's cryptographic parameters are configurable without architectural redesign: the BCrypt cost factor is an application configuration parameter, the JWT algorithm can be reconfigured within the JWT library (e.g., swapping HS256 for RS256 by changing the signing key and algorithm identifier), and TLS cipher suite selection is an infrastructure-level configuration. A documented crypto agility plan — defining the upgrade path and re-hashing migration procedure for each algorithm in the event of a cryptographic break — is being added to the security architecture documentation.</t>
+          <t>Crypto agility migration procedures documented in Documentation/CryptographicInventory.md §3. Five migration paths documented: RS256-&gt;ES256 (Keycloak key provider swap, no Spring code change), BCrypt-&gt;Argon2id (Keycloak password policy swap, transparent re-hash on login), BCrypt work-factor increase (Keycloak realm settings only), activation key size 128-&gt;256 bit (change new byte[16] to new byte[32] + Flyway migration), TLS protocol/cipher change (application.properties + nginx config). No algorithm is embedded in business logic; all changes require only configuration.</t>
         </is>
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/WebServerTlsConfig.java (configurable ENABLED_TLS_PROTOCOLS, APPROVED_CIPHER_SUITES); Security/SecurityConfig.java</t>
+          <t>Documentation/CryptographicInventory.md §3 (Migration Procedures 3.1-3.5)</t>
         </is>
       </c>
     </row>
@@ -8961,17 +8961,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>ArcadeHaven defines its logging inventory across RNF-07 and the LM-001/002/003 control catalog. The events to be logged are enumerated: authentication attempts (success and failure), authorization failures, role changes by administrators, invoice download access, activation key access, input validation failures, and security control failures. The application emits structured JSON logs to stdout. Log centralisation to an external system is an infrastructure concern outside the application layer.</t>
+          <t>Formal logging inventory documented in Documentation/LoggingInventory.md. Covers all 8 security event types (LOGIN_SUCCESS, REGISTRATION_SUCCESS, REGISTRATION_FAILURE, UNAUTHORIZED, ACCESS_DENIED, RATE_LIMIT_EXCEEDED, VALIDATION_FAILURE, ADMIN_ACTION, THRESHOLD_EXCEEDED), structured JSON format spec with all fields, dual-destination architecture (console + rolling file), access controls (appuser:appgroup, chmod 750), 30-day retention policy, explicit list of what is NOT logged (JWTs, activation keys, request bodies), and SIEM integration guidance.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityAuditService.java (SECURITY_AUDIT logger, SECURITY_EVENT/ALERT events); application.properties (logging.file.name, logging.level.SECURITY_AUDIT)</t>
+          <t>Documentation/LoggingInventory.md; Api/src/main/java/isep/desosfs/arcadehaven/Security/SecurityAuditService.java; Api/src/main/resources/logback-spring.xml</t>
         </is>
       </c>
     </row>
@@ -9179,17 +9179,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>SC-002 explicitly prohibits logging of JWT tokens, passwords, API keys, and credit card numbers in any log entry. The structured JSON log schema (LM-001) uses named fields, and IV-003 applies JSON encoding before any user-controlled value is written to a log record. A data classification table mapping each ArcadeHaven data category — password hashes, JWT tokens, activation keys, email addresses, order IDs — to an explicit logging rule (log as-is, log masked, omit entirely) is being formalized to complement the SC-002 prohibitions.</t>
+          <t>SecurityAuditService.sanitize() now applies two regex patterns before any value is embedded in a log line: JWT_PATTERN replaces full JWT tokens (eyJ... format) with [JWT_REDACTED]; ACTIVATION_KEY_PATTERN replaces 32-char uppercase hex strings with [KEY_REDACTED]. Both patterns are applied automatically to every key/value pair via the json() helper. Passwords and request bodies are never passed to logging methods. Field names (not values) appear in the details field of VALIDATION_FAILURE events.</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityAuditService.java (IP and event only, no credentials); Service/AuthService.java (username in log.error, password never logged)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Security/SecurityAuditService.java:sanitize() (JWT_PATTERN, ACTIVATION_KEY_PATTERN)</t>
         </is>
       </c>
     </row>
@@ -9453,17 +9453,17 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G17" s="21" t="inlineStr">
         <is>
-          <t>ArcadeHaven logs are emitted to stdout within the Docker container (RNF-21/22). Container-level isolation restricts direct filesystem access to the log stream to authorised operators with Docker host access. File-system access controls — read restricted to log analysis roles, write restricted to the application process, and append-only mode for the container log output — are being defined as part of the Docker deployment configuration.</t>
+          <t>Log directory /app/logs created in Dockerfile with chmod 750 and owned by appuser:appgroup (non-root container user). Only the application process can write logs; group and world have no write access. logback-spring.xml configures rolling file appender to /app/logs/arcadehaven.log with daily rotation, 30-day retention and 500 MB total cap. Container isolation prevents other processes from accessing the log volume.</t>
         </is>
       </c>
       <c r="H17" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/resources/application.properties (logging.file.name=logs/arcadehaven.log; persistent file-based log)</t>
+          <t>Api/Dockerfile (mkdir /app/logs, chmod 750); Api/src/main/resources/logback-spring.xml (RollingFileAppender)</t>
         </is>
       </c>
     </row>
@@ -9587,17 +9587,17 @@
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G21" s="21" t="inlineStr">
         <is>
-          <t>ArcadeHaven integrates with the RAWG API for game metadata enrichment (RF-12). RNF-16 defines fallback behaviour to locally stored metadata when the external API is unavailable. The circuit breaker pattern — returning cached local metadata rather than propagating raw external error responses to the client or silently skipping security checks — is being designed as part of the external integration architecture. RAWG API failures must produce a structured fallback response (abuse case AC-19).</t>
+          <t>logback-spring.xml configures dual-destination logging: CONSOLE appender (stdout, always available) and FILE appender (rolling file) with &lt;prudent&gt;true&lt;/prudent&gt;. If the file appender fails (disk full, permission error), Logback suppresses the error internally and the application continues operating via the console appender. Both appenders are attached to the root logger and the dedicated SECURITY_AUDIT logger, so security events are never silently lost.</t>
         </is>
       </c>
       <c r="H21" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Exception/GlobalExceptionHandler.java (independent @ExceptionHandler chain; error responses continue if logging fails)</t>
+          <t>Api/src/main/resources/logback-spring.xml (&lt;prudent&gt;true&lt;/prudent&gt; on RollingFileAppender, dual CONSOLE+FILE destinations)</t>
         </is>
       </c>
     </row>
@@ -14895,17 +14895,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>The application must document how rate limiting, anti-automation, and adaptive response mechanisms are applied to authentication endpoints, particularly the login and registration flows.</t>
+          <t>Rate limiting: RateLimitFilter applies Bucket4j token-bucket (20 req/min per IP) to all endpoints. No account lockout - only throttling - preventing malicious account lockout while defending against brute force. Threshold alerting: SecurityAuditService.checkAndAlert() fires SECURITY_ALERT when any IP exceeds 10 security events/60s. HIBP, context blocklist, and common-password checks are documented and enforced in PasswordPolicyService.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/RateLimitFilter.java (Bucket4j, 20 req/min per IP); Security/SecurityAuditService.java (alert threshold at 10 events/window)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Security/RateLimitFilter.java (Bucket4j 20 req/min); Security/SecurityAuditService.java (checkAndAlert); Service/PasswordPolicyService.java</t>
         </is>
       </c>
     </row>
@@ -14935,17 +14935,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>The application must maintain and enforce a list of context-specific words (e.g. "ArcadeHaven", "pixel", "vault", "admin") that cannot be used as passwords or as part of passwords.</t>
+          <t>Context-specific blocklist documented and enforced in PasswordPolicyService.CONTEXT_BLOCKLIST (21+ terms: arcadehaven, arcade, haven, pixelvault, pixel, vault, gaming, gamer, games, game, admin, password, letmein, welcome, qwerty, monkey, dragon, master, superman, batman, trustno, iloveyou, sunshine). Case-insensitive substring match applied at registration and password change.</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/PasswordPolicyService.java (CONTEXT_BLOCKLIST: arcadehaven, arcade, haven, gaming, admin, gamer, password, etc.)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/PasswordPolicyService.java:CONTEXT_BLOCKLIST, checkContextTerms()</t>
         </is>
       </c>
     </row>
@@ -14975,17 +14975,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>All authentication pathways must be documented together with their associated security controls. ArcadeHaven's JWT-based authentication flow must include documentation of token issuance, validation, expiration, and revocation mechanisms.</t>
+          <t>Single authentication pathway: POST /api/auth/login (username+password -&gt; Keycloak ROPC -&gt; JWT). All subsequent requests authenticate via JWT (Spring Security OAuth2 Resource Server). Logout (POST /api/auth/logout) revokes all Keycloak sessions. Registration (POST /api/auth/register) creates user in Keycloak and assigns role. SecurityConfig enforces JWT on all endpoints except login/register. No undocumented or backdoor pathways exist.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/AuthService.java (login, register, logout flows); Controller/AuthController.java; Security/SecurityConfig.java</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/AuthService.java (login, register, logout); Security/SecurityConfig.java (JWT validation, deny-all default)</t>
         </is>
       </c>
     </row>
@@ -15033,17 +15033,17 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>The application must enforce a minimum password length of 12 characters for all user-set passwords, validated server-side on registration and password change.</t>
+          <t>RegisterRequest enforces @Size(min=12, max=128) on password, exceeding the ASVS minimum of 8 characters. Validated server-side by Bean Validation. Same constraint enforced at Keycloak realm level.</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Dto/Request/RegisterRequest.java (@Size(min=12, max=128) on password field)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Dto/Request/RegisterRequest.java (@Size(min=12, max=128))</t>
         </is>
       </c>
     </row>
@@ -15073,17 +15073,17 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
-          <t>The application must provide all authenticated users with the ability to change their own password through a dedicated and secured endpoint.</t>
+          <t>PATCH /api/profile/password endpoint implemented in ProfileController, delegating to ProfileService.changePassword(). Requires JWT authentication. Accepts ChangePasswordRequest (currentPassword, newPassword). Verifies current password against Keycloak before applying change. Enforces full password policy on new password.</t>
         </is>
       </c>
       <c r="H8" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Controller/ProfileController.java (@PatchMapping /api/profile); Service/ProfileService.java (updateProfile)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Controller/ProfileController.java:changePassword(); Service/ProfileService.java:changePassword(); Dto/Request/ChangePasswordRequest.java</t>
         </is>
       </c>
     </row>
@@ -15113,15 +15113,19 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>The password change endpoint must require the user's current password and new password. The current password must be verified before the change is applied.</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="n"/>
+          <t>ProfileService.changePassword() calls verifyCurrentPassword() which performs a Keycloak ROPC token request with the supplied current password. If Keycloak returns 4xx, BusinessException("Current password is incorrect") is thrown and the change is rejected. Only after successful verification is the new password set via Keycloak admin API (resetPassword).</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/ProfileService.java:verifyCurrentPassword(), changePassword()</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="105" customHeight="1" s="33">
       <c r="A10" s="19" t="inlineStr">
@@ -15149,17 +15153,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
-          <t>The application must check all passwords submitted during registration or password change against a blocklist of at least the top 3000 most common passwords. Passwords found on the blocklist must be rejected with an appropriate error message.</t>
+          <t>PasswordPolicyService.checkCommonPasswords() checks submitted passwords against top-3000+ common passwords loaded from /security/common-passwords.txt (case-insensitive). Called at registration and password change.</t>
         </is>
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/PasswordPolicyService.java (checkHibp: k-anonymity SHA-1 prefix HIBP check; checkCommonPasswords: 3000+ blocked passwords)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/PasswordPolicyService.java:checkCommonPasswords(); src/main/resources/security/common-passwords.txt</t>
         </is>
       </c>
     </row>
@@ -15189,17 +15193,17 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>The application must not impose character composition rules on passwords. No requirement for uppercase, lowercase, numbers, or special characters shall be enforced. Only minimum length will be validated.</t>
+          <t>PasswordPolicyService.validate() enforces only: minimum length, context blocklist, common password list, and HIBP breach check. No composition rules - no uppercase/lowercase/digit/special character requirements. Any Unicode character combination accepted. RegisterRequest and ChangePasswordRequest use @Size only.</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/PasswordPolicyService.java (only length/blocklist/HIBP checks enforced, no character composition restrictions)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/PasswordPolicyService.java (no composition checks); Dto/Request/RegisterRequest.java (@Size only)</t>
         </is>
       </c>
     </row>
@@ -15341,17 +15345,17 @@
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>The application must permit passwords of at least 64 characters in length. The database schema and all validation layers must support this without truncation.</t>
+          <t>RegisterRequest and ChangePasswordRequest both enforce @Size(min=12, max=128). The 128-character maximum exceeds the 64-character minimum. Keycloak realm policy configured consistently.</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Dto/Request/RegisterRequest.java (@Size(max=128) allows passwords up to 128 chars)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Dto/Request/RegisterRequest.java (@Size(max=128)); Dto/Request/ChangePasswordRequest.java (@Size(max=128))</t>
         </is>
       </c>
     </row>
@@ -15381,17 +15385,17 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>The application must not enforce periodic password expiration. Passwords remain valid until the user changes them voluntarily or a breach is detected.</t>
+          <t>No periodic password expiration enforced. Keycloak realm has no force-expired-password-change policy. Passwords remain valid until voluntarily changed by the user or a breach is detected (HIBP).</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/AuthService.java (Keycloak manages password lifecycle); Config/KeycloakAdminConfig.java</t>
+          <t>Keycloak realm: no password expiry policy; Api/src/main/java/isep/desosfs/arcadehaven/Service/AuthService.java (no expiry enforcement)</t>
         </is>
       </c>
     </row>
@@ -15421,17 +15425,17 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
-          <t>The application must actively validate passwords against the context-specific blocklist defined in previously during registration and password change, rejecting any password that contains a blocked term.</t>
+          <t>PasswordPolicyService.checkContextTerms() performs case-insensitive substring search against CONTEXT_BLOCKLIST at registration (AuthService.register()) and password change (ProfileService.changePassword()). Rejection message is generic and does not disclose the matched term.</t>
         </is>
       </c>
       <c r="H17" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/PasswordPolicyService.java (checkContextSpecific: blocklist enforced at registration)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/PasswordPolicyService.java:checkContextTerms()</t>
         </is>
       </c>
     </row>
@@ -15461,17 +15465,17 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>The application must check passwords submitted during registration and password changes against a breached password database. The HaveIBeenPwned API (k-anonymity model) will be used to perform this check without exposing the plain-text password.</t>
+          <t>PasswordPolicyService.checkHibp() computes SHA-1, sends 5-char prefix to HaveIBeenPwned k-anonymity API, checks if suffix appears in response. Full hash never transmitted. Applied at registration and password change. Configurable via security.hibp.enabled=false for offline environments.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/PasswordPolicyService.java (checkHibp: Have I Been Pwned k-anonymity integration)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/PasswordPolicyService.java:checkHibp()</t>
         </is>
       </c>
     </row>
@@ -15599,17 +15603,17 @@
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G22" s="16" t="inlineStr">
         <is>
-          <t>The application must support multi-factor authentication. MFA must be mandatory for ADMIN role accounts and optional for PUBLISHER and BUYER roles. TOTP (RFC 6238) is the target mechanism.</t>
+          <t>MFA delegated to Keycloak. Keycloak supports TOTP (RFC 6238, 6-digit, 30-second step) as second factor. MFA is mandatory for ADMIN accounts via Keycloak required action CONFIGURE_TOTP on admin users. BUYER and PUBLISHER can optionally enrol via Keycloak account console. The Spring Boot API validates the JWT issued by Keycloak after successful MFA completion.</t>
         </is>
       </c>
       <c r="H22" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/AuthService.java (Keycloak MFA delegation); Config/KeycloakAdminConfig.java</t>
+          <t>Keycloak realm: MFA / TOTP required action for ADMIN; Api/src/main/java/isep/desosfs/arcadehaven/Config/KeycloakAdminConfig.java</t>
         </is>
       </c>
     </row>
@@ -15639,17 +15643,17 @@
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G23" s="21" t="inlineStr">
         <is>
-          <t>All authentication pathways must be documented and subject to the same security controls. No undocumented or backdoor authentication pathways are permitted.</t>
+          <t>ArcadeHaven has a single documented authentication pathway (V6.1.3). SecurityConfig applies JWT validation uniformly to all secured endpoints. No endpoint bypasses JWT except explicitly permitted /api/auth/login and /api/auth/register. No undocumented or test-only authentication bypasses exist.</t>
         </is>
       </c>
       <c r="H23" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/AuthService.java (login/register/logout); Security/SecurityConfig.java (consistent JWT validation across all endpoints)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Security/SecurityConfig.java (uniform JWT, deny-all default)</t>
         </is>
       </c>
     </row>
@@ -15825,17 +15829,17 @@
       </c>
       <c r="F29" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>System-generated passwords and activation codes must be generated using a cryptographically secure random number generator (SecureRandom), comply with the password policy, and expire within 24 hours of generation.</t>
+          <t>Game activation keys (system-generated secrets) use SecureRandom.nextBytes(16) (128-bit CSPRNG) encoded as 32-char hex. Activation keys are single-use: consumed on first redemption via OrderItem.redeem(). Initial admin password is provided via ADMIN_PASSWORD env var (not system-generated). No default passwords.</t>
         </is>
       </c>
       <c r="H29" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Config/AdminInitializer.java (env-var ADMIN_PASSWORD for initial admin account)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Domain/OrderItem.java:generateActivationKey() (SecureRandom 128-bit); Config/AdminInitializer.java (ADMIN_PASSWORD env var)</t>
         </is>
       </c>
     </row>
@@ -15905,15 +15909,19 @@
       </c>
       <c r="F31" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G31" s="16" t="inlineStr">
         <is>
-          <t>The password reset process must use a cryptographically secure, single-use token with a maximum validity of 1 hour. The process must not bypass MFA and must invalidate the token immediately after use.</t>
-        </is>
-      </c>
-      <c r="H31" s="16" t="n"/>
+          <t>Password reset handled entirely by Keycloak: sends time-limited (5 min), single-use secure email link. Reset link invalidated immediately after use. Does not bypass MFA. No custom reset flow in Spring Boot.</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Keycloak realm: forgot-password flow (5-min single-use token via secure email)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="60" customHeight="1" s="33">
       <c r="A32" s="19" t="inlineStr">
@@ -15941,15 +15949,19 @@
       </c>
       <c r="F32" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G32" s="21" t="inlineStr">
         <is>
-          <t>Account recovery following loss of an MFA factor must require identity verification at the same assurance level as the original enrollment process.</t>
-        </is>
-      </c>
-      <c r="H32" s="21" t="n"/>
+          <t>MFA factor recovery handled by Keycloak Admin Console: admin removes TOTP credential and sets CONFIGURE_TOTP as required action, forcing re-enrolment at same assurance level as original enrolment. No self-service MFA recovery bypass in the application.</t>
+        </is>
+      </c>
+      <c r="H32" s="21" t="inlineStr">
+        <is>
+          <t>Keycloak Admin Console: Users -&gt; Credentials -&gt; remove OTP -&gt; required action CONFIGURE_TOTP</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1" s="33">
       <c r="A33" s="14" t="inlineStr">
@@ -16059,15 +16071,19 @@
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>All one-time passwords, lookup secrets, and out-of-band codes must be invalidated immediately after a single successful use. Replay of used codes must be rejected.</t>
-        </is>
-      </c>
-      <c r="H36" s="16" t="n"/>
+          <t>TOTP codes single-use by design: Keycloak maintains used-code cache preventing replay within same time window. Password reset tokens single-use: invalidated after first use. Activation keys single-use: consumed on redemption via OrderItem.redeem().</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>Keycloak TOTP: used-code cache (anti-replay); Api/src/main/java/isep/desosfs/arcadehaven/Domain/OrderItem.java:redeem()</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="90" customHeight="1" s="33">
       <c r="A37" s="19" t="inlineStr">
@@ -16095,15 +16111,19 @@
       </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G37" s="21" t="inlineStr">
         <is>
-          <t>All lookup secrets stored in the database must be hashed using BCrypt or an equivalent approved password hashing algorithm. Plain-text storage of any secret is strictly prohibited.</t>
-        </is>
-      </c>
-      <c r="H37" s="21" t="n"/>
+          <t>TOTP seeds stored by Keycloak in AES-encrypted credential store (not accessible to Spring Boot). Activation keys have 128-bit entropy (&gt;= 112 bits), so a standard hash is permitted by ASVS; they are stored as display-once values access-controlled at DB level.</t>
+        </is>
+      </c>
+      <c r="H37" s="21" t="inlineStr">
+        <is>
+          <t>Keycloak credential store (AES-encrypted TOTP seeds); Api/src/main/java/isep/desosfs/arcadehaven/Domain/OrderItem.java (128-bit activation key, display-once)</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="105" customHeight="1" s="33">
       <c r="A38" s="14" t="inlineStr">
@@ -16131,15 +16151,19 @@
       </c>
       <c r="F38" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>All lookup secrets, out-of-band authentication codes, and TOTP seeds must be generated using SecureRandom or an equivalent CSPRNG. Use of Math.random() or similar non-cryptographic generators is strictly prohibited.</t>
-        </is>
-      </c>
-      <c r="H38" s="16" t="n"/>
+          <t>TOTP seeds and password reset tokens generated by Keycloak using SecureRandom. Activation keys generated via java.security.SecureRandom.nextBytes(16) in OrderItem.generateActivationKey(). No Math.random() or non-cryptographic generator used in any secret-generation path.</t>
+        </is>
+      </c>
+      <c r="H38" s="16" t="inlineStr">
+        <is>
+          <t>Keycloak (SecureRandom for TOTP seeds and reset tokens); Api/src/main/java/isep/desosfs/arcadehaven/Domain/OrderItem.java:generateActivationKey() (SecureRandom)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="105" customHeight="1" s="33">
       <c r="A39" s="19" t="inlineStr">
@@ -16167,15 +16191,19 @@
       </c>
       <c r="F39" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G39" s="21" t="inlineStr">
         <is>
-          <t>All lookup secrets and out-of-band authentication codes must have a minimum of 20 bits of entropy. ArcadeHaven will use 6-character alphanumeric codes as the baseline, providing at least 31 bits of entropy.</t>
-        </is>
-      </c>
-      <c r="H39" s="21" t="n"/>
+          <t>Keycloak TOTP generates 6-digit codes (log2(10^6) ~20 bits of entropy, meets 20-bit minimum). Password reset tokens &gt;= 128 bits. Activation keys 128 bits. No code falls below 20-bit threshold.</t>
+        </is>
+      </c>
+      <c r="H39" s="21" t="inlineStr">
+        <is>
+          <t>Keycloak TOTP: 6-digit codes (~20 bits); Activation keys: 128 bits</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="75" customHeight="1" s="33">
       <c r="A40" s="14" t="inlineStr">
@@ -16203,15 +16231,19 @@
       </c>
       <c r="F40" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>Out-of-band authentication codes must expire after a maximum of 5 minutes. TOTP validation must use a time window of ±1 step (30 seconds). Expired codes must be rejected.</t>
-        </is>
-      </c>
-      <c r="H40" s="16" t="n"/>
+          <t>Keycloak TOTP: 30-second time step with +/-1 step tolerance (90 sec max window, within 30s requirement). Password reset links expire after 5 minutes (within 10-minute max for out-of-band requests). Email verification codes expire after 5 minutes.</t>
+        </is>
+      </c>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>Keycloak realm: OTP Policy (30s step, +/-1 tolerance); action-token-generated-by-admin-lifespan=5m</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="30" customHeight="1" s="33">
       <c r="A41" s="19" t="inlineStr">
@@ -16389,15 +16421,19 @@
       </c>
       <c r="F46" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G46" s="21" t="inlineStr">
         <is>
-          <t>All out-of-band authentication codes must be cryptographically bound to the specific authentication request and session for which they were generated. Cross-session reuse must be rejected.</t>
-        </is>
-      </c>
-      <c r="H46" s="21" t="n"/>
+          <t>Keycloak TOTP codes time-bound (30s) and session-scoped. Used-code tracking prevents replay in different sessions. Password reset tokens cryptographically bound to specific user and action; cannot be used for different user or action.</t>
+        </is>
+      </c>
+      <c r="H46" s="21" t="inlineStr">
+        <is>
+          <t>Keycloak TOTP: session-scoped, used-code tracking; Keycloak reset tokens: user-ID-bound, single-use</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="72" customHeight="1" s="33">
       <c r="A47" s="14" t="inlineStr">
@@ -16425,15 +16461,19 @@
       </c>
       <c r="F47" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G47" s="16" t="inlineStr">
         <is>
-          <t>OTP verification endpoints must enforce rate limiting, rejecting further attempts after 5 consecutive failures. Codes must expire after a maximum of 5 minutes as defined in V6.5.5.</t>
-        </is>
-      </c>
-      <c r="H47" s="16" t="n"/>
+          <t>Keycloak brute force protection enabled: increasing wait time after consecutive MFA failures, permanent lockout after threshold. RateLimitFilter additionally limits all requests (including login/MFA) to 20 req/min per IP as secondary layer. TOTP codes expire after 30 seconds limiting brute-force window.</t>
+        </is>
+      </c>
+      <c r="H47" s="16" t="inlineStr">
+        <is>
+          <t>Keycloak realm: brute-force protection; Api/src/main/java/isep/desosfs/arcadehaven/Security/RateLimitFilter.java (20 req/min, secondary layer)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="30" customHeight="1" s="33">
       <c r="A48" s="19" t="inlineStr">
@@ -16669,17 +16709,17 @@
       </c>
       <c r="F55" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>JWT access tokens must have a maximum validity of 15 minutes. A token denylist mechanism must be implemented to support immediate invalidation upon logout or security events.</t>
+          <t>JWT access tokens: Keycloak access-token-lifespan configured to 900 seconds (15 minutes). Session revocation: AuthService.logout() calls keycloak.realm().users().get(userId).logout() immediately invalidating all active Keycloak sessions. Spring Security validates JWT on every request against Keycloak JWKS endpoint. Note: ASVS V6.8.3 text references SAML assertions; observation correctly applies JWT token validity controls in this context.</t>
         </is>
       </c>
       <c r="H55" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/AuthService.java (logout() calls keycloak.realm().users().get().logout() revoking all sessions); Controller/AuthController.java</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/AuthService.java:logout() (Keycloak session revocation); Keycloak realm: access-token-lifespan=900s (15 min)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Implementation of the Security Vulnerability & Architecture Risk Policy on the application #3 #9
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -8017,17 +8017,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>This is a Level 3 requirement. ArcadeHaven targets ASVS Level 2. Spring beans are singletons by default; thread-safety depends on all service and controller components being stateless. A formal thread-safety audit of all shared state has not been performed.</t>
+          <t>Formal SLA documented: Critical CVEs &lt;=7 days, High &lt;=30 days, Medium &lt;=90 days, Low next release. OWASP Dependency Check runs on every CI execution (sca-dependency-check.yml). False-positive suppression procedure defined.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Api/pom.xml (owasp dependency-check-maven plugin); .github/workflows/sast-codeql.yml (CodeQL security-extended); .github/workflows/sca-dependency-check.yml</t>
+          <t>Documentation/VulnerabilityRemediationPolicy.md §1; .github/workflows/sca-dependency-check.yml</t>
         </is>
       </c>
     </row>
@@ -8057,17 +8057,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>pom.xml provides a complete list of all direct third-party dependencies. All dependencies are sourced from Maven Central, a pre-defined and trusted repository. A formal SBOM in CycloneDX format is being generated via the cyclonedx-maven-plugin, which includes transitive dependencies.</t>
+          <t>CycloneDX SBOM generated on every build (cyclonedx:makeAggregateBom, build.yml). bom.xml and bom.json uploaded as report-build-test artifact. All dependencies from Maven Central (trusted repository).</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>Api/pom.xml (cyclonedx-maven-plugin 2.9.0); .github/workflows/build.yml (makeAggregateBom + artifact upload)</t>
+          <t>Api/pom.xml (cyclonedx-maven-plugin 2.9.0); .github/workflows/build.yml</t>
         </is>
       </c>
     </row>
@@ -8097,17 +8097,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Resource-demanding operations identified and documented: file uploads (FO-001/002 — max size and MIME validation), PDF invoice generation via iText (RF-16/26 — triggered only on confirmed order completion), and RAWG API calls (RF-12/RNF-16 — configurable timeout with local metadata fallback). Rate limiting (AC-006, RNF-09) applies across all high-volume endpoints.</t>
+          <t>Resource-demanding functionality formally documented: file uploads (25 MB cap, Tika MIME check), SFTP operations (SSH host-key verification), HIBP check (fail-open), invoice/key-card generation, Keycloak Admin API calls, DB game-listing (composite indexes). Each entry lists risk and mitigations.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>Api/pom.xml (all dependencies explicitly versioned via Spring Boot BOM)</t>
+          <t>Documentation/VulnerabilityRemediationPolicy.md §2</t>
         </is>
       </c>
     </row>
@@ -8169,17 +8169,17 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Although a Level 3 requirement, ArcadeHaven's V15.1.3 analysis already identifies and documents all resource-demanding and high-risk functionality: file uploads (disk I/O, MIME validation bypass risk), PDF invoice generation via iText (server-side file generation with user-controlled order data), RAWG API HTTP calls (SSRF adjacency, external dependency), and activation key generation (CSPRNG entropy dependency). These represent the dangerous functionality areas. A separate formal "dangerous functionality" section is being added to the security architecture documentation to satisfy the explicit V15.1.5 framing.</t>
+          <t>8 dangerous features formally labelled with risk category and mitigations: file upload (path traversal, MIME spoofing), RAWG SSRF adjacency, Keycloak Admin API, ROPC grant, admin initialisation, JWT signing keys, SFTP host-key, activation keys.</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>Api/pom.xml (maven-checkstyle-plugin, spotbugs-maven-plugin, owasp dependency-check); .github/workflows/code-quality.yml; .github/workflows/sast-codeql.yml</t>
+          <t>Documentation/VulnerabilityRemediationPolicy.md §3</t>
         </is>
       </c>
     </row>
@@ -8227,17 +8227,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Dependencies are version-pinned in pom.xml. OWASP Dependency Check is being integrated into the CI/CD pipeline to scan all direct and transitive dependencies against the NVD on each build, blocking any component with a CVE that exceeds the documented remediation timeframe (V15.1.1). No known high or critical CVEs have been identified in the current dependency set.</t>
+          <t>OWASP Dependency Check (dependency-check-maven 12.1.3) runs on every CI execution against NVD database with NVD_API_KEY secret. Build fails on CVE threshold breach. Report uploaded as report-sca artifact. Remediation SLA enforces no components past timeframe in production.</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>Api/pom.xml (Spring Boot 4.0.6, Spring Security, Keycloak 26.0.5, sshj 0.38.0 - all actively maintained)</t>
+          <t>.github/workflows/sca-dependency-check.yml; Api/pom.xml; Documentation/VulnerabilityRemediationPolicy.md §1</t>
         </is>
       </c>
     </row>
@@ -8477,17 +8477,17 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>The only outbound HTTP call in ArcadeHaven is to the RAWG API for game metadata enrichment (RF-12). The HTTP client (RestTemplate or WebClient) is explicitly configured to disable automatic redirect-following. An unexpected redirect from the RAWG API is treated as a failure and falls back to locally stored metadata (RNF-16).</t>
+          <t>RestTemplate bean configured with anonymous SimpleClientHttpRequestFactory subclass that overrides prepareConnection() calling connection.setInstanceFollowRedirects(false). Applied to all outbound HTTP calls: AuthService (ROPC login/logout) and ProfileService (current-password verification). Future RAWG client inherits this bean.</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/AuthService.java (Keycloak Admin API with BusinessException wrapping); Service/SftpStorageService.java (SFTP with StorageException wrapping)</t>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Config/KeycloakAdminConfig.java</t>
         </is>
       </c>
     </row>
@@ -8557,17 +8557,17 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>The Docker deployment configuration is defining the reverse proxy layer to forward the original client IP via the X-Forwarded-For header. The application reads the client IP from this trusted header for rate limiting (AC-006) and security event logging (LM-001). The proxy configuration strips any client-supplied X-Forwarded-For headers before appending its own, preventing IP spoofing at the application boundary.</t>
+          <t>server.forward-headers-strategy=NATIVE activates Tomcat RemoteIpFilter. server.tomcat.remoteip.trusted-proxies restricts trust to RFC-1918 ranges (Docker networks). Client-supplied X-Forwarded-For headers are stripped. RateLimitFilter and SecurityEventHandler use request.getRemoteAddr() directly.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Exception/GlobalExceptionHandler.java (resolveClientIp handles X-Forwarded-For); Security/SecurityConfig.java</t>
+          <t>Api/src/main/resources/application.properties; Api/src/main/java/isep/desosfs/arcadehaven/Security/RateLimitFilter.java; SecurityEventHandler.java</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Integration of OAuthGrantConfigTest and improvement of SecurityAuditService and correction of testes #9 #12 #13
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -453,7 +453,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -632,7 +632,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -809,7 +809,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -984,7 +984,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1159,7 +1159,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1210,7 +1210,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1240,7 +1240,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -3768,12 +3768,12 @@
       </c>
       <c r="G19" s="21" t="inlineStr">
         <is>
-          <t>Implicit flow (response_type=token) is explicitly disabled for all ArcadeHaven clients (implicitFlowEnabled=false). However, the Resource Owner Password Credentials grant is used by AuthService.login() as an architectural dependency -- the Spring Boot API acts as a login proxy for clients that cannot perform browser redirects. PKCE Authorization Code flow is enforced for browser clients.</t>
+          <t>Implicit Flow explicitly disabled (implicitFlowEnabled=false). Direct Access Grant (ROPC) retained as an architectural dependency — ArcadeHaven has no frontend SPA, so Authorization Code + PKCE redirect is not yet feasible. Formally documented as DEV-01 in Documentation/SecurityDeviations.md with business justification, residual risk, and 11 compensating controls (rate limiting, brute-force protection, short token lifetime, single-use refresh tokens, MFA for admins, session revocation, full audit logging, HTTPS, PKCE pre-configured). 6 automated tests in OAuthGrantConfigTest verify these controls. Planned remediation: disable Direct Access Grant when frontend SPA is added.</t>
         </is>
       </c>
       <c r="H19" s="21" t="inlineStr">
         <is>
-          <t>keycloak/realm-export.json (arcadehaven-public: implicitFlowEnabled=false); Api/src/main/.../Service/AuthService.java (login() uses Direct Grant -- architectural dependency)</t>
+          <t>Documentation/SecurityDeviations.md (DEV-01); keycloak/realm-export.json; Api/src/main/java/.../Service/AuthService.java; Api/src/test/.../Config/OAuthGrantConfigTest.java</t>
         </is>
       </c>
     </row>
@@ -6519,17 +6519,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>All communication channels will be documented, including database connectivity, external API integration and server-side file generation</t>
+          <t>All application communication channels documented in Documentation/CommunicationMatrix.md. Lists 5 external connections (PostgreSQL, SFTP/SSH, ClamAV, HaveIBeenPwned k-anonymity API, RAWG future) and 5 internal Docker connections (nginx-&gt;app, app-&gt;Keycloak, Keycloak-&gt;DB, inbound HTTPS, inbound HTTP redirect). Each entry documents: direction, protocol, port, authentication method, data sensitivity level (L1-L4), TLS status, and source file reference. TLS posture summary and required actions included.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Api/docker-compose.yml (inter-service network: api, keycloak, postgres, sftp-server); application.properties (all external service endpoints documented)</t>
+          <t>Documentation/CommunicationMatrix.md</t>
         </is>
       </c>
     </row>
@@ -7403,17 +7403,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>All sensitive data in ArcadeHaven will be identified and classified. Key sensitive data includes: password hashes, JWT tokens, activation keys, personal user data (email, username), order history, and payment-related data. JWT payloads will be treated as sensitive despite being only Base64-encoded. Classification will be documented in the data protection policy.</t>
+          <t>Formal data classification document created: Documentation/DataClassificationPolicy.md. Defines 4 levels (L1 Public, L2 Internal, L3 Confidential, L4 Restricted). Maps all ArcadeHaven data types: game metadata (L1), audit logs (L2), user PII / JWT tokens / activation keys / orders (L3), password hashes / client secrets / DB credentials (L4). Specifies controls per level (access control, logging restrictions, transport, storage, retention). Includes retention schedule: audit logs 30 days, JWT access 5 min, refresh 30 days, user data until deletion.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Service/PasswordPolicyService.java (SHA-1 prefix only for HIBP, full hash never stored); Security/SecurityAuditService.java (IP logged, no credentials)</t>
+          <t>Documentation/DataClassificationPolicy.md</t>
         </is>
       </c>
     </row>
@@ -7537,17 +7537,17 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G7" s="21" t="inlineStr">
         <is>
-          <t>Sensitive API responses will include Cache-Control: no-store headers to prevent caching in intermediary layers such as load balancers or reverse proxies.</t>
+          <t>SecurityConfig.java sets Cache-Control: no-cache, no-store, max-age=0, must-revalidate and Pragma: no-cache on all API responses via .cacheControl(Customizer.withDefaults()), preventing intermediary caching of sensitive data. Verified by SecurityHeadersTest.</t>
         </is>
       </c>
       <c r="H7" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Exception/GlobalExceptionHandler.java (generic error messages only, no internal details leaked); Security/SecurityEventHandler.java</t>
+          <t>Api/src/main/java/.../Security/SecurityConfig.java; Api/src/test/.../Security/SecurityHeadersTest.java</t>
         </is>
       </c>
     </row>
@@ -7622,12 +7622,12 @@
       </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
-          <t>Controls defined in V14.1.2 will be implemented and verified: BCrypt for password hashing, TLS for data in transit, Cache-Control: no-store for sensitive responses, role-based access to sensitive log data, and data retention policies enforced via scheduled database cleanup jobs.</t>
+          <t>BCrypt hashing (via Keycloak) ✅. Log redaction enforced: SecurityAuditService.json() automatically redacts any field whose key matches SENSITIVE_KEY_PATTERN (password/secret/credential/private_key/client_secret); sanitize() also strips form-encoded credentials (password=value). Data retention formally documented in DataClassificationPolicy.md §4 (logs 30d, JWT 5min, refresh 30d). Remaining gap: DB TLS (sslmode=require) pending on remote PostgreSQL server TLS enablement. 7 new unit tests in SecurityAuditServiceTest validate redaction behaviour.</t>
         </is>
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/resources/application.properties (TLS config); Security/WebServerTlsConfig.java; Security/SecurityConfig.java</t>
+          <t>Api/src/main/java/.../Security/SecurityAuditService.java (SENSITIVE_KEY_PATTERN); Documentation/DataClassificationPolicy.md; Api/src/test/.../Security/SecurityAuditServiceTest.java</t>
         </is>
       </c>
     </row>
@@ -7839,17 +7839,17 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>Sensitive responses include Cache-Control: no-store to prevent caching by browsers, proxies, and intermediaries.</t>
+          <t>Same Cache-Control implementation as V14.2.2: SecurityConfig.java applies no-store, no-cache headers globally via cacheControl(Customizer.withDefaults()), preventing browser caching of tokens, user data, and activation keys. Verified by SecurityHeadersTest.</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityConfig.java (.cacheControl(Customizer.withDefaults()) sets Cache-Control: no-cache, no-store)</t>
+          <t>Api/src/main/java/.../Security/SecurityConfig.java; Api/src/test/.../Security/SecurityHeadersTest.java</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement ASVS V9.2.2/V9.2.3/V9.2.4 - JWT typ and audience claim validation #9 #12 #13
Add JwtBearerTypValidator to reject non-Bearer token types (ID/Refresh tokens), wire custom JwtDecoder in SecurityConfig with typ + aud validators, and add missing jwt.audiences=arcadehaven-api property to enforce audience claim validation that was previously documented but never enforced. Fix JwtAudienceConfigTest to assert the audiences property instead of the issuer-uri.
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -453,7 +453,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -545,7 +545,7 @@
                   <v>0.5</v>
                 </pt>
                 <pt idx="4">
-                  <v>0.75</v>
+                  <v>1</v>
                 </pt>
                 <pt idx="5">
                   <v>0.8461538461538461</v>
@@ -566,7 +566,7 @@
                   <v>1</v>
                 </pt>
                 <pt idx="11">
-                  <v>0</v>
+                  <v>0.6666666666666666</v>
                 </pt>
                 <pt idx="12">
                   <v>1</v>
@@ -632,7 +632,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -721,7 +721,7 @@
                   <v>0</v>
                 </pt>
                 <pt idx="3">
-                  <v>0.125</v>
+                  <v>0.375</v>
                 </pt>
                 <pt idx="4">
                   <v>0.8</v>
@@ -745,13 +745,13 @@
                   <v>0.8181818181818182</v>
                 </pt>
                 <pt idx="11">
-                  <v>0</v>
+                  <v>0.5</v>
                 </pt>
                 <pt idx="12">
-                  <v>0.25</v>
+                  <v>0.3333333333333333</v>
                 </pt>
                 <pt idx="13">
-                  <v>0.1428571428571428</v>
+                  <v>0.5714285714285714</v>
                 </pt>
                 <pt idx="14">
                   <v>0.9</v>
@@ -809,7 +809,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -984,7 +984,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1073,10 +1073,10 @@
                   <v>0.09677419354838709</v>
                 </pt>
                 <pt idx="3">
-                  <v>0.125</v>
+                  <v>0.25</v>
                 </pt>
                 <pt idx="4">
-                  <v>0.5384615384615384</v>
+                  <v>0.6153846153846154</v>
                 </pt>
                 <pt idx="5">
                   <v>0.6382978723404256</v>
@@ -1097,13 +1097,13 @@
                   <v>0.5833333333333334</v>
                 </pt>
                 <pt idx="11">
-                  <v>0</v>
+                  <v>0.4166666666666667</v>
                 </pt>
                 <pt idx="12">
-                  <v>0.1904761904761905</v>
+                  <v>0.2380952380952381</v>
                 </pt>
                 <pt idx="13">
-                  <v>0.1538461538461539</v>
+                  <v>0.3846153846153846</v>
                 </pt>
                 <pt idx="14">
                   <v>0.6666666666666666</v>
@@ -1159,7 +1159,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1210,7 +1210,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1240,7 +1240,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -2991,17 +2991,17 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
-          <t>ArcadeHaven will issue distinct token types (access token, refresh token)</t>
+          <t>ASVS V9.2.2 — JwtBearerTypValidator (Security/JwtBearerTypValidator.java) implements OAuth2TokenValidator&lt;Jwt&gt; that rejects any token whose typ claim is present and not Bearer (case-insensitive). Fail-open for tokens without typ to support all Keycloak versions. Wired into custom JwtDecoder bean in SecurityConfig.jwtDecoder() via DelegatingOAuth2TokenValidator alongside issuer and audience validators. 6 unit tests in JwtBearerTypValidatorTest validate: Bearer accepted, case-insensitive, missing typ accepted, ID rejected, Refresh rejected, arbitrary type rejected.</t>
         </is>
       </c>
       <c r="H8" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityConfig.java (Spring Security JWT decoder validates exp, nbf, iss automatically)</t>
+          <t>Api/src/main/java/.../Security/JwtBearerTypValidator.java; Api/src/main/java/.../Security/SecurityConfig.java (jwtDecoder bean); Api/src/test/java/.../Security/JwtBearerTypValidatorTest.java (6 tests)</t>
         </is>
       </c>
     </row>
@@ -3031,17 +3031,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>JWT tokens will include an aud (audience) claim set to arcadehaven-api. The validation layer will reject any token whose aud claim does not match the expected value.</t>
+          <t>ASVS V9.2.3 — spring.security.oauth2.resourceserver.jwt.audiences=arcadehaven-api added to application.properties. SecurityConfig.jwtDecoder() bean adds JwtClaimValidator&lt;List&lt;String&gt;&gt; for the aud claim, requiring arcadehaven-api to be present. Keycloak client arcadehaven-public has oidc-audience-mapper that adds arcadehaven-api to aud on every access token. Any token missing this value is rejected with 401. 4 tests in JwtAudienceConfigTest verify the property configuration.</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityConfig.java (issuer-uri validation per realm); application.properties (jwk-set-uri)</t>
+          <t>Api/src/main/resources/application.properties (audiences=arcadehaven-api); Api/src/main/java/.../Security/SecurityConfig.java (JwtClaimValidator aud); Api/src/test/java/.../Config/JwtAudienceConfigTest.java (4 tests)</t>
         </is>
       </c>
     </row>
@@ -3071,17 +3071,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
-          <t>ArcadeHaven uses a single audience (arcadehaven-api), so audience confusion risk is low.</t>
+          <t>ASVS V9.2.4 — Single fixed audience arcadehaven-api eliminates audience confusion: tokens issued for any other Keycloak client are rejected by the JwtClaimValidator in SecurityConfig.jwtDecoder(). No dynamic audience provisioning. Audience restriction enforced at both Keycloak (oidc-audience-mapper) and Spring Security (JwtClaimValidator) layers — defence in depth.</t>
         </is>
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityConfig.java (JWK set URI bound to single Keycloak realm); application.properties (jwt.issuer-uri)</t>
+          <t>Api/src/main/resources/application.properties (audiences=arcadehaven-api); Api/src/main/java/.../Security/SecurityConfig.java (jwtDecoder bean); keycloak/realm-export.json (oidc-audience-mapper)</t>
         </is>
       </c>
     </row>
@@ -13623,17 +13623,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>All HTTP traffic is redirected to HTTPS at the reverse proxy level. The application itself is only exposed over HTTPS.</t>
+          <t>In the development environment, the API is exposed locally over HTTP only and is not publicly available. HTTPS is to be enforced in production environments here TLS is terminated at a reserve proxy (Nginx/Traefik), responsible for enforcing TSL 1.2+ and reedirecting non-HTTPS traffic to the correct endpoints.</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/RateLimitFilter.java (Bucket4j, 20 req/min per IP on /api/auth/login, /api/auth/register, /api/publisher/games)</t>
+          <t>Api/src/main/resource/application.properties</t>
         </is>
       </c>
     </row>
@@ -13663,17 +13663,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Headers such as `X-Real-IP` and `X-Forwarded-For` set by intermediary layers (e.g. reverse proxy, Docker network) will be validated server-side. End-users will not be able to override these headers. Configuration will be enforced in the Spring Boot application and documented in the deployment guide.</t>
+          <t>ArcadeHaven application odes not trust client-provided headers such as X-Forwarded-For, X-Real-IP or X-Forwarded-Proto. These headers are only allowed hen injected through trusted reversse proxies. Additionally, SpringBoot is configured to ensure fowarded headers are only accepted from known internal proxy range and all other application componentes rely on request.getRemoteAddr() after proxy resolution.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityConfig.java; Security/RateLimitFilter.java; Dto/Request/ (Bean Validation annotations)</t>
+          <t>Api/src/main/resources/application.properties; Api/src/main/.../Security/SecurityAuditService.java;  Api/src/main/…/Exception/GlobalExceptionHandler.java; Api/src/main/…/Security/SecurityAuditService.java</t>
         </is>
       </c>
     </row>
@@ -14405,7 +14405,7 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G6" s="21" t="inlineStr">

</xml_diff>

<commit_message>
tests: Improvement of the Unit Tests to have the Coverage Report on 84% of coverage and creation of the K6 tests to verify the load, the availability and the response time of the application #12 #13
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -453,7 +453,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -632,7 +632,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -809,7 +809,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -984,7 +984,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1159,7 +1159,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1210,7 +1210,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1240,7 +1240,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -11538,7 +11538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="33" min="1" max="1"/>
@@ -12083,10 +12083,14 @@
       </c>
       <c r="F17" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G17" s="29" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G17" s="29" t="inlineStr">
+        <is>
+          <t>RateLimitFilter covers /api/auth/login and /api/auth/register (20 req/min per IP). High-risk endpoints not yet covered: POST /api/publisher/games, POST /api/orders/{id}/complete, POST /api/library/import-key. Extend filter with per-endpoint Bucket4j buckets.</t>
+        </is>
+      </c>
       <c r="H17" s="16" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1" s="33">
@@ -12120,6 +12124,804 @@
       </c>
       <c r="G18" s="30" t="n"/>
       <c r="H18" s="21" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>V7.1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Session Management Documentation</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>V7.1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Session Management Documentation</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>V7.1.1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Verify that the session inactivity timeout and absolute maximum lifetime are documented.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>JWT access token lifetime controlled by Keycloak. No formal document defines and justifies these values (NIST SP 800-63B). Action: verify Keycloak Realm Settings → Tokens values (Access Token Lifespan, Client Session Idle) and document them.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Keycloak Realm Settings → Tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>V7.1</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Session Management Documentation</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>V7.1.2</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Verify that concurrent session limits and the behavior when exceeded are documented.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Stateless JWT design allows unlimited concurrent sessions by default. This design decision (no concurrent session limit) must be explicitly documented and justified.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Architectural decision — stateless JWT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>V7.1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Session Management Documentation</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>V7.1.3</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Verify that requirements around federated identity session management, such as how SSO session expiry relates to the application session expiry, are documented.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No documentation covers how Keycloak SSO session lifetime relates to individual JWT lifetimes and what triggers re-authentication.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Keycloak SSO config</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>V7.3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Session Timeout</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>V7.3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Session Timeout</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>V7.3.1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Verify that the session inactivity timeout is enforced and the user is required to re-authenticate when this timeout is reached.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>JWT access token has a TTL (Keycloak → Realm Settings → Tokens → Access Token Lifespan). Client Session Idle (refresh token invalidated if unused for N minutes) acts as inactivity timeout. Action: verify values are &lt;= 15 min access / &lt;= 7 days refresh idle, and document.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Keycloak Realm Settings → Tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>V7.3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Session Timeout</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>V7.3.2</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Verify that an absolute maximum session lifetime is enforced, after which re-authentication is required regardless of session activity.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Client Session Max in Keycloak defines the absolute maximum before forced re-authentication. Action: verify it is &lt;= 7 days (604800 s) per ASVS V10.4.8, and document.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Keycloak → Client Session Max</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>V7.4</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Session Termination</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>V7.4</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Session Termination</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>V7.4.2</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Verify that all sessions are terminated when a user account is disabled or deleted.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>AdminService.deactivateUser() sets the active flag in DB but does NOT call UserResource.logout() on Keycloak. Active JWT sessions remain valid until expiry. Fix: call authService.logout(userId) immediately after deactivation.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/AdminService.java</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>V7.4</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Session Termination</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>V7.4.3</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Verify that users have the option to terminate all other active sessions after a successful password change or factor change.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Keycloak can revoke all sessions on password change via Realm Settings → Security Defences → Revoke Refresh Tokens. PATCH /api/profile/password calls Keycloak Admin API to change credential; whether sessions are revoked depends on realm config. Action: verify and document.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Keycloak realm config</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>V7.4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Session Termination</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>V7.4.5</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Verify that administrators can terminate active sessions for individual users or all users.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>No endpoint in AdminController exposes session revocation. AuthService.logout(username) already contains the logic. Fix: add DELETE /api/admin/users/{id}/sessions that resolves the user Keycloak ID and calls UserResource.logout().</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Controller/AdminController.java</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>V7.5</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Re-authentication for Sensitive Operations</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>V7.5</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Re-authentication for Sensitive Operations</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>V7.5.1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Verify that changing the user's authentication credentials requires re-authentication.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Password change (PATCH /api/profile/password) already requires currentPassword. Email change (PATCH /api/profile) does NOT require re-authentication — a stolen JWT can change the account email. Fix: add optional currentPassword to UpdateProfileRequest and require it when email is changing.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Dto/Request/UpdateProfileRequest.java</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>V7.5</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Re-authentication for Sensitive Operations</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>V7.5.2</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Verify that users can view and terminate any or all of their current active sessions and authenticated devices.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Keycloak Account Console (/realms/arcadehaven/account) allows any authenticated user to view and revoke active sessions. No Spring Boot endpoint provides this capability directly. Action: document this path; optionally expose GET /api/profile/sessions proxy endpoint.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>/realms/arcadehaven/account (Keycloak Account Console)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>V7.6</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Session Management for Federated Identity</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>V7.6</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Session Management for Federated Identity</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>V7.6.1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Verify that the session lifetime and termination behavior between relying party and identity provider is documented.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Spring Boot (RP) uses stateless JWTs; Keycloak (IdP) manages the SSO session. When a JWT expires, the client refreshes via the refresh token. If the Keycloak session is forcibly terminated, previously issued JWTs remain valid until exp. POST /api/auth/logout revokes Keycloak sessions explicitly. This behaviour needs to be formally documented.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/AuthService.java</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>V13.2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Backend Component Authentication</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>V13.2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Backend Component Authentication</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>V13.2.1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Verify that all backend component communications use the principle of short-lived credentials (e.g., short-lived tokens, certificates, and secrets).</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Keycloak Admin Client uses OAuth2 client credentials flow (short-lived tokens). SFTP uses SSH key. PostgreSQL uses a static username/password — no rotation or certificate-based auth. Full compliance requires migrating DB auth to a vault-managed rotating credential or client certificate.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Api/src/main/resources/application.properties (spring.datasource.url)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>V13.2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Backend Component Authentication</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>V13.2.2</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Verify that backend components use only the minimum necessary level of access to external services, datastores, and secrets.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>The PostgreSQL user has full access to all tables. Flyway (DDL) and the application (DML) should use separate database users: one with CREATE TABLE/ALTER TABLE for migrations, one with only SELECT/INSERT/UPDATE/DELETE for the application.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Api/docker-compose.yml (DB service); Api/src/main/resources/application.properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>V13.2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Backend Component Authentication</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>V13.2.4</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Verify that an allowlist is used to define permitted external resources and systems that the application is permitted to use.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>The application connects to Keycloak, PostgreSQL, SFTP, and HIBP. No explicit egress allowlist is enforced at the network layer. Mitigation: document all permitted egress destinations; add Docker network rules; fix RAWG base URL as a code constant when implemented.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Api/docker-compose.yml (networks config)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>V13.3</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Secrets Management</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>V13.3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Secrets Management</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>V13.3.1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Verify that a secrets management solution such as a key vault is used to create, store, and control access to secrets.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Secrets (DB_PASSWORD, KEYCLOAK_CLIENT_SECRET, ADMIN_PASSWORD, SFTP_PRIVATE_KEY_PATH) are provided via a .env file. Acceptable for development/CI but inadequate for production. Target: Docker Secrets or Kubernetes Secret / HashiCorp Vault. .env is excluded from the Docker image via .dockerignore.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Api/.dockerignore; Api/docker-compose.yml (env_file)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>V13.3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Secrets Management</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>V13.3.2</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Verify that access to secrets follows the principle of least privilege, such that the service only has access to the secrets it needs.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>With the current .env approach, all secrets are visible to any process in the same container — no per-secret access control. Remediation depends on V13.3.1 (vault or Docker Secrets). Blocked until V13.3.1 is resolved.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Depends on V13.3.1</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F18">

</xml_diff>

<commit_message>
database: Flyway migration implementation #4 #10 #11
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -11538,7 +11538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="33" min="1" max="1"/>
@@ -12136,12 +12136,6 @@
           <t>Session Management Documentation</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -12280,12 +12274,6 @@
           <t>Session Timeout</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -12382,12 +12370,6 @@
           <t>Session Termination</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -12526,12 +12508,6 @@
           <t>Re-authentication for Sensitive Operations</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -12628,12 +12604,6 @@
           <t>Session Management for Federated Identity</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -12688,12 +12658,6 @@
           <t>Backend Component Authentication</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -12765,17 +12729,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>The PostgreSQL user has full access to all tables. Flyway (DDL) and the application (DML) should use separate database users: one with CREATE TABLE/ALTER TABLE for migrations, one with only SELECT/INSERT/UPDATE/DELETE for the application.</t>
+          <t>spring.flyway.url/user/password configured with FLYWAY_DATASOURCE_* env-var overrides. In dev/CI falls back to main datasource. In production: create DDL-only user for Flyway and DML-only for the app, then set FLYWAY_DATASOURCE_URL/USERNAME/PASSWORD env vars.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Api/docker-compose.yml (DB service); Api/src/main/resources/application.properties</t>
+          <t>Api/src/main/resources/application.properties (Flyway section); Api/docker-compose.yml (comment)</t>
         </is>
       </c>
     </row>
@@ -12832,12 +12796,6 @@
           <t>Secrets Management</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -12920,6 +12878,174 @@
       <c r="H41" t="inlineStr">
         <is>
           <t>Depends on V13.3.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>V12.2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Secure Communication</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>V12.2.2</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Verify that a publicly trusted TLS certificate is used in production.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>nginx reverse proxy uses self-signed cert for dev/CI. Production deployments must replace nginx/certs/server.crt and server.key with a cert from Let's Encrypt or institutional CA — one-file swap, no code change needed.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Api/nginx/nginx.conf; Api/nginx/generate-self-signed-cert.sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>V12.3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Secure Communication</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>V12.3.1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Verify that all inbound and outbound connections use TLS.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>SFTP uses SSH. sslmode=prefer now active via spring.datasource.hikari.data-source-properties.sslmode=\. Change DB_SSL_MODE=require in .env once remote DB has TLS enabled. Nginx-to-app link uses HTTP within Docker bridge (single-host, acceptable).</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Api/src/main/resources/application.properties (HIKARICP section)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>V12.3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Secure Communication</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>V12.3.3</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Verify that all intra-service communications are encrypted.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Docker bridge network is not encrypted. For production mTLS between all containers, deploy with Kubernetes + service mesh (Istio/Linkerd) or Docker Swarm encrypted overlay network.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Api/docker-compose.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>V14.2</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Data Protection</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>V14.2.4</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Verify that controls appropriate to the data classification are implemented.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>BCrypt hashing, log sanitization, data retention all compliant. sslmode=prefer active via HikariCP (DB_SSL_MODE env var). Full compliance requires DB_SSL_MODE=require once remote DB at vsgate-s1.dei.isep.ipp.pt:10345 has TLS enabled.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Api/src/main/resources/application.properties (HIKARICP section); Documentation/DataClassificationPolicy.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Implementation of deactivate all user sessions and deactivate user account #9 #10
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <sheet name="V17 - WebRTC" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="181029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -736,7 +736,7 @@
                   <v>0.3333333333333333</v>
                 </pt>
                 <pt idx="8">
-                  <v>0</v>
+                  <v>1</v>
                 </pt>
                 <pt idx="9">
                   <v>0.75</v>
@@ -1088,7 +1088,7 @@
                   <v>0.3076923076923077</v>
                 </pt>
                 <pt idx="8">
-                  <v>0.5714285714285714</v>
+                  <v>1</v>
                 </pt>
                 <pt idx="9">
                   <v>0.6111111111111112</v>
@@ -11538,7 +11538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="33" min="1" max="1"/>
@@ -12125,930 +12125,6 @@
       <c r="G18" s="30" t="n"/>
       <c r="H18" s="21" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>V7.1</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Session Management Documentation</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>V7.1</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Session Management Documentation</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>V7.1.1</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Verify that the session inactivity timeout and absolute maximum lifetime are documented.</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>JWT access token lifetime controlled by Keycloak. No formal document defines and justifies these values (NIST SP 800-63B). Action: verify Keycloak Realm Settings → Tokens values (Access Token Lifespan, Client Session Idle) and document them.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Keycloak Realm Settings → Tokens</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>V7.1</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Session Management Documentation</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>V7.1.2</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Verify that concurrent session limits and the behavior when exceeded are documented.</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Stateless JWT design allows unlimited concurrent sessions by default. This design decision (no concurrent session limit) must be explicitly documented and justified.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Architectural decision — stateless JWT</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>V7.1</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Session Management Documentation</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>V7.1.3</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Verify that requirements around federated identity session management, such as how SSO session expiry relates to the application session expiry, are documented.</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>No documentation covers how Keycloak SSO session lifetime relates to individual JWT lifetimes and what triggers re-authentication.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Keycloak SSO config</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>V7.3</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Session Timeout</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>V7.3</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Session Timeout</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>V7.3.1</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Verify that the session inactivity timeout is enforced and the user is required to re-authenticate when this timeout is reached.</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>JWT access token has a TTL (Keycloak → Realm Settings → Tokens → Access Token Lifespan). Client Session Idle (refresh token invalidated if unused for N minutes) acts as inactivity timeout. Action: verify values are &lt;= 15 min access / &lt;= 7 days refresh idle, and document.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Keycloak Realm Settings → Tokens</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>V7.3</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Session Timeout</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>V7.3.2</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Verify that an absolute maximum session lifetime is enforced, after which re-authentication is required regardless of session activity.</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Client Session Max in Keycloak defines the absolute maximum before forced re-authentication. Action: verify it is &lt;= 7 days (604800 s) per ASVS V10.4.8, and document.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Keycloak → Client Session Max</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>V7.4</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Session Termination</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>V7.4</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Session Termination</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>V7.4.2</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Verify that all sessions are terminated when a user account is disabled or deleted.</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>AdminService.deactivateUser() sets the active flag in DB but does NOT call UserResource.logout() on Keycloak. Active JWT sessions remain valid until expiry. Fix: call authService.logout(userId) immediately after deactivation.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/AdminService.java</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>V7.4</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Session Termination</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>V7.4.3</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Verify that users have the option to terminate all other active sessions after a successful password change or factor change.</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Keycloak can revoke all sessions on password change via Realm Settings → Security Defences → Revoke Refresh Tokens. PATCH /api/profile/password calls Keycloak Admin API to change credential; whether sessions are revoked depends on realm config. Action: verify and document.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Keycloak realm config</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>V7.4</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Session Termination</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>V7.4.5</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Verify that administrators can terminate active sessions for individual users or all users.</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>No endpoint in AdminController exposes session revocation. AuthService.logout(username) already contains the logic. Fix: add DELETE /api/admin/users/{id}/sessions that resolves the user Keycloak ID and calls UserResource.logout().</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Api/src/main/java/isep/desosfs/arcadehaven/Controller/AdminController.java</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>V7.5</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Re-authentication for Sensitive Operations</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>V7.5</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Re-authentication for Sensitive Operations</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>V7.5.1</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Verify that changing the user's authentication credentials requires re-authentication.</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Password change (PATCH /api/profile/password) already requires currentPassword. Email change (PATCH /api/profile) does NOT require re-authentication — a stolen JWT can change the account email. Fix: add optional currentPassword to UpdateProfileRequest and require it when email is changing.</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Api/src/main/java/isep/desosfs/arcadehaven/Dto/Request/UpdateProfileRequest.java</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>V7.5</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Re-authentication for Sensitive Operations</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>V7.5.2</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Verify that users can view and terminate any or all of their current active sessions and authenticated devices.</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Keycloak Account Console (/realms/arcadehaven/account) allows any authenticated user to view and revoke active sessions. No Spring Boot endpoint provides this capability directly. Action: document this path; optionally expose GET /api/profile/sessions proxy endpoint.</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>/realms/arcadehaven/account (Keycloak Account Console)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>V7.6</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Session Management for Federated Identity</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>V7.6</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Session Management for Federated Identity</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>V7.6.1</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Verify that the session lifetime and termination behavior between relying party and identity provider is documented.</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Spring Boot (RP) uses stateless JWTs; Keycloak (IdP) manages the SSO session. When a JWT expires, the client refreshes via the refresh token. If the Keycloak session is forcibly terminated, previously issued JWTs remain valid until exp. POST /api/auth/logout revokes Keycloak sessions explicitly. This behaviour needs to be formally documented.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Api/src/main/java/isep/desosfs/arcadehaven/Service/AuthService.java</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>V13.2</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Backend Component Authentication</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>V13.2</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Backend Component Authentication</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>V13.2.1</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Verify that all backend component communications use the principle of short-lived credentials (e.g., short-lived tokens, certificates, and secrets).</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Keycloak Admin Client uses OAuth2 client credentials flow (short-lived tokens). SFTP uses SSH key. PostgreSQL uses a static username/password — no rotation or certificate-based auth. Full compliance requires migrating DB auth to a vault-managed rotating credential or client certificate.</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Api/src/main/resources/application.properties (spring.datasource.url)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>V13.2</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Backend Component Authentication</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>V13.2.2</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Verify that backend components use only the minimum necessary level of access to external services, datastores, and secrets.</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>spring.flyway.url/user/password configured with FLYWAY_DATASOURCE_* env-var overrides. In dev/CI falls back to main datasource. In production: create DDL-only user for Flyway and DML-only for the app, then set FLYWAY_DATASOURCE_URL/USERNAME/PASSWORD env vars.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Api/src/main/resources/application.properties (Flyway section); Api/docker-compose.yml (comment)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>V13.2</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Backend Component Authentication</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>V13.2.4</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Verify that an allowlist is used to define permitted external resources and systems that the application is permitted to use.</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>The application connects to Keycloak, PostgreSQL, SFTP, and HIBP. No explicit egress allowlist is enforced at the network layer. Mitigation: document all permitted egress destinations; add Docker network rules; fix RAWG base URL as a code constant when implemented.</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Api/docker-compose.yml (networks config)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>V13.3</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Secrets Management</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>V13.3</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Secrets Management</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>V13.3.1</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Verify that a secrets management solution such as a key vault is used to create, store, and control access to secrets.</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Secrets (DB_PASSWORD, KEYCLOAK_CLIENT_SECRET, ADMIN_PASSWORD, SFTP_PRIVATE_KEY_PATH) are provided via a .env file. Acceptable for development/CI but inadequate for production. Target: Docker Secrets or Kubernetes Secret / HashiCorp Vault. .env is excluded from the Docker image via .dockerignore.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Api/.dockerignore; Api/docker-compose.yml (env_file)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>V13.3</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Secrets Management</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>V13.3.2</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Verify that access to secrets follows the principle of least privilege, such that the service only has access to the secrets it needs.</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>With the current .env approach, all secrets are visible to any process in the same container — no per-secret access control. Remediation depends on V13.3.1 (vault or Docker Secrets). Blocked until V13.3.1 is resolved.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Depends on V13.3.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>V12.2</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Secure Communication</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>V12.2.2</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Verify that a publicly trusted TLS certificate is used in production.</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>nginx reverse proxy uses self-signed cert for dev/CI. Production deployments must replace nginx/certs/server.crt and server.key with a cert from Let's Encrypt or institutional CA — one-file swap, no code change needed.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Api/nginx/nginx.conf; Api/nginx/generate-self-signed-cert.sh</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>V12.3</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Secure Communication</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>V12.3.1</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Verify that all inbound and outbound connections use TLS.</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>SFTP uses SSH. sslmode=prefer now active via spring.datasource.hikari.data-source-properties.sslmode=\. Change DB_SSL_MODE=require in .env once remote DB has TLS enabled. Nginx-to-app link uses HTTP within Docker bridge (single-host, acceptable).</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Api/src/main/resources/application.properties (HIKARICP section)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>V12.3</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Secure Communication</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>V12.3.3</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Verify that all intra-service communications are encrypted.</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Docker bridge network is not encrypted. For production mTLS between all containers, deploy with Kubernetes + service mesh (Istio/Linkerd) or Docker Swarm encrypted overlay network.</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Api/docker-compose.yml</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>V14.2</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Data Protection</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>V14.2.4</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Verify that controls appropriate to the data classification are implemented.</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>BCrypt hashing, log sanitization, data retention all compliant. sslmode=prefer active via HikariCP (DB_SSL_MODE env var). Full compliance requires DB_SSL_MODE=require once remote DB at vsgate-s1.dei.isep.ipp.pt:10345 has TLS enabled.</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Api/src/main/resources/application.properties (HIKARICP section); Documentation/DataClassificationPolicy.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F18">
     <cfRule type="cellIs" priority="2" operator="equal">
@@ -13061,7 +12137,7 @@
       <formula>"Not Applicable"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation sqref="F2:F1018" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Compliant,Not Applicable"</formula1>
       <formula2>0</formula2>
@@ -18289,10 +17365,14 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G16" s="21" t="n"/>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>AdminService.deactivateUser() now calls keycloakDisableAndLogout(): sets enabled=false on Keycloak user (blocks new logins) + calls UserResource.logout() (revokes all active sessions immediately). activateUser() calls keycloakEnable() to re-enable the account.</t>
+        </is>
+      </c>
       <c r="H16" s="21" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1" s="33">
@@ -18385,10 +17465,14 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G19" s="16" t="n"/>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>DELETE /api/admin/users/{id}/sessions endpoint added to AdminController. AdminService.revokeUserSessions() resolves Keycloak user by username and calls UserResource.logout() to revoke all sessions immediately without disabling the account.</t>
+        </is>
+      </c>
       <c r="H19" s="16" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1" s="33">

</xml_diff>

<commit_message>
feat: Implementation of validateSubDir and validateRemotePath on SFTP, implementation of SSRF: enforce egress allowlist on all outbound RestTemplate calls #4 #6 #9
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -10935,17 +10935,17 @@
       </c>
       <c r="F19" s="28" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G19" s="29" t="inlineStr">
         <is>
-          <t>ArcadeHaven enforces input size constraints and value bounds in Dto files and sanitizes potentially dangerous context when building invoices. Uploaded files are assigned sanitized filenames before being store in file storage</t>
+          <t>SftpStorageService.validateSubDir() rejects subdir paths containing ".." or starting with "/"; validateRemotePath() asserts download/delete paths start with baseRemoteDir and contain no "..".; sanitizeFilename() strips unsafe chars from all SFTP filenames (applied in both uploadFile() and uploadBytes()). LocalStorageService.resolveAndValidate() uses Path.normalize() + startsWith(baseDir) for the local backend. FileStorageService.sanitizeText() strips CR/LF/TAB from activation-key file content; InvoiceService.sanitizeLine() does the same for invoice lines. All RAWG-sourced strings are HTML-stripped and whitespace-normalised before persisting (see V1.1.2).</t>
         </is>
       </c>
       <c r="H19" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/java/…/Dto/Request; Api/src/main/java/…/Service/InvoiceService.java; Api/src/main/java/…/Service/FileStorageService.java; Api/main/java/…/Service/SftpStorageService.java</t>
+          <t>Api/src/main/java/.../Service/SftpStorageService.java (validateSubDir, validateRemotePath, sanitizeFilename); Service/LocalStorageService.java (resolveAndValidate); Service/FileStorageService.java (sanitizeText); Service/InvoiceService.java (sanitizeLine)</t>
         </is>
       </c>
     </row>
@@ -11047,11 +11047,19 @@
       </c>
       <c r="F22" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G22" s="30" t="n"/>
-      <c r="H22" s="21" t="n"/>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="G22" s="30" t="inlineStr">
+        <is>
+          <t>Two enforcement layers: (1) Application layer — EgressAllowlistInterceptor (ClientHttpRequestInterceptor) is wired into the shared RestTemplate bean; blocks any outbound call to a host not in the allowlist (Keycloak host from ${keycloak.server-url} + api.rawg.io). Throws IOException before the connection is made. HIBP calls use Java HttpClient with the URL hardcoded as a constant in PasswordPolicyService. (2) Docker network layer — keycloak-internal network (internal: true) isolates keycloak-db from internet and from the app container; app-services bridge provides controlled connectivity between nginx, app and keycloak for JWT verification and admin API.</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>Api/src/main/java/.../Security/EgressAllowlistInterceptor.java; Config/KeycloakAdminConfig.java (restTemplate bean — wires interceptor with allowed hosts); Api/docker-compose.yml (networks: keycloak-internal internal: true, app-services)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1" s="33">
       <c r="A23" s="14" t="inlineStr">
@@ -17911,17 +17919,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>Authorization will be based on role-based access control, defining permissions for roles</t>
+          <t>Documentation/AuthorizationMatrix.md documents all 37 API endpoints with role permissions (ADMIN, PUBLISHER, BUYER) and ownership checks. SecurityConfig.java enforces path-level rules (deny-all default). @PreAuthorize("hasRole(...)") annotations on each controller method enforce method-level authorization. Service-layer ownership checks (e.g. GameService.findByIdAndPublisher, OrderService ownership) enforce data-specific access rules.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityConfig.java (role-based URL rules: ADMIN, PUBLISHER, BUYER; deny-all default)</t>
+          <t>Documentation/AuthorizationMatrix.md (37 endpoints, role matrix, ownership rules — V8.1.1); Api/src/main/java/.../Security/SecurityConfig.java; Controller/AdminController.java, PublisherController.java, GameController.java, OrderController.java, LibraryController.java (@PreAuthorize)</t>
         </is>
       </c>
     </row>
@@ -17951,17 +17959,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>Field-level access control will be enforced at the API response layer using DTO projections and service-level filtering to prevent exposure of sensitive attributes</t>
+          <t>Documentation/AuthorizationMatrix.md §V8.1.2 documents readable and writable fields per role per entity. Sensitive fields (password_hash, activation_key, invoice_path, internal IDs) are excluded from all API responses. DTO record projections (GameResponse, OrderResponse, UserResponse, LibraryEntryResponse) enforce field-level filtering at the service layer. Publishers cannot read other publishers fields; buyers cannot read game cost price etc.</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>Api/src/main/.../Security/SecurityConfig.java; Service/GameService.java (findByIdAndPublisher); Service/FileStorageService.java (path traversal prevention)</t>
+          <t>Documentation/AuthorizationMatrix.md §V8.1.2 (field-level access table); Api/src/main/java/.../Dto/Response/GameResponse.java, OrderResponse.java, UserResponse.java, LibraryEntryResponse.java (DTO projections exclude sensitive fields)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Improvement of the endpoints of the RateLimitFilter, Testing app availability with K6 testing and docker and finalization of the ASVS Report #3 #4 #9
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\dmopm\IdeaProjects\desofs2026-wed_nap_2\Deliverables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmopm\IdeaProjects\desofs2026-wed_nap_2\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6FB5DDA-7F68-49A6-A2E5-13DE01415BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B7BE21-8113-4276-AB33-B380DCDDE8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -7478,7 +7478,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>236</v>
+        <v>1008</v>
       </c>
       <c r="G19" s="21" t="s">
         <v>797</v>

</xml_diff>